<commit_message>
solucionando cosas de las anotaciones en vergara junio/mayo
</commit_message>
<xml_diff>
--- a/BELGRANO 1646/Junio/JUNIO-BLG1646.xlsx
+++ b/BELGRANO 1646/Junio/JUNIO-BLG1646.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\OneDrive\Desktop\RC CONSORCIO 2025\BELGRANO 1646\Junio\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D44982A5-B39C-4AA8-B98F-A243AA8C48C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD6A0776-1A04-42B9-9330-1A2465DB1E60}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -19,14 +19,14 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="1">PRORRATEO!$A$1:$N$64</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">RESUMEN!$A$1:$F$146</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">RESUMEN!$A$1:$F$153</definedName>
   </definedNames>
   <calcPr calcId="181029"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="267" uniqueCount="177">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="272" uniqueCount="178">
   <si>
     <t>consorciobelgrano1640@gmail.com</t>
   </si>
@@ -480,54 +480,30 @@
     <t>FEUILLANT, GASTON</t>
   </si>
   <si>
-    <t>Ferreteria</t>
-  </si>
-  <si>
     <t>Contessi provision y colocacion de 60 lts de aceite hidraulico en la sede del monta auto</t>
   </si>
   <si>
     <t>SEGURO OBLIGATORIO SR DIEGO BRITEZ FEDERACION PATRONAL DEBITO AUTOMATICO 05/05</t>
   </si>
   <si>
-    <t>Arreglo de motor retirado y reemplazado por uno nuevo en montavehiculos</t>
-  </si>
-  <si>
     <t>Debito 12/05</t>
   </si>
   <si>
     <t>Pago mis cuentas 12/05</t>
   </si>
   <si>
-    <t>Fumigacion 12/05</t>
-  </si>
-  <si>
-    <t>Doartero Julio - Ajuste de todas las puertas y reparacion de la puerta principal 16/05</t>
-  </si>
-  <si>
     <t>Camaras del sur 19/05 - compra y colocacion camaras de entradas (pileta y gimnasio)</t>
   </si>
   <si>
-    <t>Servisur - cambio de luminarias 19/05</t>
-  </si>
-  <si>
     <t>Numero 1859135 Debito automatico 5/05</t>
   </si>
   <si>
-    <t xml:space="preserve">Antonio santillan plomero - Arreglo tanque </t>
-  </si>
-  <si>
     <t>Salvatierra limpieza de columna de baño desde piso 3 (inclusive) hasta el piso 10 (inclusive) - 20/05</t>
   </si>
   <si>
-    <t>Guido Alterini - Jardineria : Adelanto compra pasto</t>
-  </si>
-  <si>
     <t>Kromacolor  -  Compra de materiales : Sellador Sika 23/05</t>
   </si>
   <si>
-    <t>Doartero Julio - Emergencia purga de grupo electrogeno por falta de combustible 26/05</t>
-  </si>
-  <si>
     <t>Compra Fabio Tolosa - Combustible 19/05</t>
   </si>
   <si>
@@ -555,18 +531,12 @@
     <t>Reparacion puerta SUM 02/05</t>
   </si>
   <si>
-    <t>Preinstalacion nueva aire acondicionado SUM - Leandro Gomez 27/5</t>
-  </si>
-  <si>
     <t>Compra de Juan Manuel Villa - Combustible 23/05</t>
   </si>
   <si>
     <t>Debito 27/05</t>
   </si>
   <si>
-    <t>Gabriel Villegas - Envio carte documento Edesur</t>
-  </si>
-  <si>
     <t>ADS - Imputado en el mes de Marzo y transferido finalizada las charlas por la desvinculacion</t>
   </si>
   <si>
@@ -592,6 +562,39 @@
   </si>
   <si>
     <t>Ingreso mes de MAYO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kromacolor </t>
+  </si>
+  <si>
+    <t>Contessi</t>
+  </si>
+  <si>
+    <t>Servisur - cambio de luminarias 18/06</t>
+  </si>
+  <si>
+    <t>Fumigacion 10/06</t>
+  </si>
+  <si>
+    <t>SA seguridad - 10/06 - Servicio tecnico realizado en motor de porton, se lubrica caja reductora</t>
+  </si>
+  <si>
+    <t>Zaffalon Veronica - Por vaciamiento de monta coches con agua y mucho residuo de aceite, extraido con bomba y balde por la pesadez de lo econtrado</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Servisur </t>
+  </si>
+  <si>
+    <t>Eba - Elcetrica de buenos aires</t>
+  </si>
+  <si>
+    <t>Casa ruan - materiales de trabajo</t>
+  </si>
+  <si>
+    <t>Ferreteria Arcamone - Yeso de 5 kilos</t>
+  </si>
+  <si>
+    <t>Presupuesto 18/06</t>
   </si>
 </sst>
 </file>
@@ -1319,7 +1322,7 @@
     <xf numFmtId="167" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="255">
+  <cellXfs count="260">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="34" xfId="0" applyBorder="1"/>
@@ -1622,6 +1625,21 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="13" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1700,15 +1718,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -1718,68 +1727,69 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="35" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="36" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="35" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="36" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="37" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="31" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="33" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="5" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="15" fillId="5" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="35" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="36" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="5" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="5" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="37" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="5" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="20" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -2146,7 +2156,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:N156"/>
+  <dimension ref="A1:N163"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="33.42578125" customWidth="1"/>
@@ -2156,7 +2166,8 @@
     <col min="5" max="5" width="15.7109375" customWidth="1"/>
     <col min="6" max="6" width="13" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="15.85546875" customWidth="1"/>
-    <col min="8" max="9" width="13" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="14.85546875" customWidth="1"/>
+    <col min="9" max="9" width="13" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="14.5703125" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="18" customWidth="1"/>
     <col min="13" max="13" width="18.28515625" customWidth="1"/>
@@ -2203,10 +2214,10 @@
         <v>1</v>
       </c>
       <c r="B5" s="71" t="s">
-        <v>170</v>
+        <v>160</v>
       </c>
       <c r="C5" s="71" t="s">
-        <v>169</v>
+        <v>159</v>
       </c>
       <c r="D5" s="71"/>
       <c r="E5" s="72"/>
@@ -2234,26 +2245,26 @@
     <row r="11" spans="1:5" hidden="1" x14ac:dyDescent="0.25"/>
     <row r="12" spans="1:5" hidden="1" x14ac:dyDescent="0.25"/>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="B14" s="202" t="s">
+      <c r="B14" s="207" t="s">
         <v>135</v>
       </c>
-      <c r="C14" s="203"/>
-      <c r="D14" s="204"/>
+      <c r="C14" s="208"/>
+      <c r="D14" s="209"/>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="B15" s="205"/>
-      <c r="C15" s="206"/>
-      <c r="D15" s="207"/>
+      <c r="B15" s="210"/>
+      <c r="C15" s="211"/>
+      <c r="D15" s="212"/>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="B16" s="205"/>
-      <c r="C16" s="206"/>
-      <c r="D16" s="207"/>
+      <c r="B16" s="210"/>
+      <c r="C16" s="211"/>
+      <c r="D16" s="212"/>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="B17" s="208"/>
-      <c r="C17" s="209"/>
-      <c r="D17" s="210"/>
+      <c r="B17" s="213"/>
+      <c r="C17" s="214"/>
+      <c r="D17" s="215"/>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19" s="3"/>
@@ -2278,7 +2289,7 @@
         <v>16</v>
       </c>
       <c r="B22" s="7" t="s">
-        <v>171</v>
+        <v>161</v>
       </c>
       <c r="C22" s="7"/>
       <c r="D22" s="130"/>
@@ -2341,7 +2352,7 @@
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A26" s="121" t="s">
-        <v>159</v>
+        <v>151</v>
       </c>
       <c r="B26" s="7"/>
       <c r="C26" s="7"/>
@@ -2710,7 +2721,7 @@
     </row>
     <row r="52" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A52" s="94" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="B52" s="7"/>
       <c r="C52" s="98"/>
@@ -2732,20 +2743,20 @@
         <v>5</v>
       </c>
       <c r="B53" s="7" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="C53" s="7"/>
-      <c r="D53" s="113">
-        <f>102143.27+6011.02+54099.18</f>
-        <v>162253.47</v>
+      <c r="D53" s="256">
+        <f>55568.88+6174.32+104266.16</f>
+        <v>166009.35999999999</v>
       </c>
       <c r="E53" s="134">
         <f>D53*91.91%</f>
-        <v>149127.16427699997</v>
+        <v>152579.20277599996</v>
       </c>
       <c r="F53" s="134">
         <f>D53*8.09%</f>
-        <v>13126.305722999999</v>
+        <v>13430.157223999999</v>
       </c>
       <c r="H53" s="150"/>
     </row>
@@ -2753,20 +2764,20 @@
       <c r="A54" s="94" t="s">
         <v>136</v>
       </c>
-      <c r="B54" s="7" t="s">
-        <v>144</v>
+      <c r="B54" s="258" t="s">
+        <v>142</v>
       </c>
       <c r="C54" s="7"/>
-      <c r="D54" s="113">
-        <v>532295.61</v>
+      <c r="D54" s="256">
+        <v>546846.93999999994</v>
       </c>
       <c r="E54" s="134">
         <f>D54*91.91%</f>
-        <v>489232.89515099995</v>
+        <v>502607.02255399991</v>
       </c>
       <c r="F54" s="134">
         <f>D54*8.09%</f>
-        <v>43062.714848999996</v>
+        <v>44239.917445999992</v>
       </c>
       <c r="H54" s="150"/>
     </row>
@@ -2778,19 +2789,19 @@
       <c r="C55" s="96"/>
       <c r="D55" s="108">
         <f>SUM(D52:D54)</f>
-        <v>699569.08</v>
+        <v>717876.29999999993</v>
       </c>
       <c r="E55" s="108">
         <f t="shared" ref="E55:F55" si="7">SUM(E52:E54)</f>
-        <v>642973.94142799987</v>
+        <v>659800.10732999991</v>
       </c>
       <c r="F55" s="108">
         <f t="shared" si="7"/>
-        <v>56595.138571999996</v>
+        <v>58076.192669999989</v>
       </c>
       <c r="G55" s="109">
         <f>E55+F55</f>
-        <v>699569.07999999984</v>
+        <v>717876.29999999993</v>
       </c>
       <c r="H55" s="150" t="str">
         <f>IF(D55=G55, "", "Error")</f>
@@ -2810,7 +2821,7 @@
     </row>
     <row r="57" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A57" s="114" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B57" s="176"/>
       <c r="C57" s="177"/>
@@ -2845,157 +2856,153 @@
       </c>
       <c r="B58" s="176"/>
       <c r="C58" s="177"/>
-      <c r="D58" s="113">
-        <v>330000</v>
+      <c r="D58" s="256">
+        <v>1350000</v>
       </c>
       <c r="E58" s="149">
         <f>D58</f>
-        <v>330000</v>
+        <v>1350000</v>
       </c>
       <c r="F58" s="7"/>
       <c r="G58" s="109">
         <f>D58</f>
-        <v>330000</v>
+        <v>1350000</v>
       </c>
       <c r="H58" s="161">
         <f>E58+F58</f>
-        <v>330000</v>
+        <v>1350000</v>
       </c>
       <c r="I58" s="178">
-        <f t="shared" ref="I58:I86" si="11">H58-D58</f>
+        <f t="shared" ref="I58:I93" si="11">H58-D58</f>
         <v>0</v>
       </c>
       <c r="J58" s="178">
-        <f t="shared" ref="J58:J86" si="12">G58-D58</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="59" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A59" s="121" t="s">
+        <f t="shared" ref="J58:J93" si="12">G58-D58</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59" spans="1:10" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A59" s="190" t="s">
+        <v>168</v>
+      </c>
+      <c r="B59" s="176"/>
+      <c r="C59" s="177"/>
+      <c r="D59" s="256">
+        <v>5000</v>
+      </c>
+      <c r="E59" s="149">
+        <f>D59</f>
+        <v>5000</v>
+      </c>
+      <c r="F59" s="7"/>
+      <c r="G59" s="109">
+        <f>D59</f>
+        <v>5000</v>
+      </c>
+      <c r="H59" s="161">
+        <f>E59+F59</f>
+        <v>5000</v>
+      </c>
+      <c r="I59" s="178">
+        <f>H59-D59</f>
+        <v>0</v>
+      </c>
+      <c r="J59" s="178"/>
+    </row>
+    <row r="60" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A60" s="121" t="s">
         <v>8</v>
       </c>
-      <c r="B59" s="163"/>
-      <c r="C59" s="7"/>
-      <c r="D59" s="113">
-        <v>143638</v>
-      </c>
-      <c r="E59" s="149">
-        <f t="shared" ref="E59:E63" si="13">D59*91.91%</f>
-        <v>132017.68579999998</v>
-      </c>
-      <c r="F59" s="134">
-        <f t="shared" ref="F59:F63" si="14">D59*8.09%</f>
-        <v>11620.314200000001</v>
-      </c>
-      <c r="G59" s="109">
-        <f t="shared" ref="G59:G86" si="15">D59</f>
-        <v>143638</v>
-      </c>
-      <c r="H59" s="161">
-        <f t="shared" ref="H59:H86" si="16">E59+F59</f>
-        <v>143637.99999999997</v>
-      </c>
-      <c r="I59" s="178">
-        <f t="shared" si="11"/>
-        <v>0</v>
-      </c>
-      <c r="J59" s="178">
-        <f t="shared" si="12"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="60" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A60" s="94" t="s">
-        <v>172</v>
-      </c>
-      <c r="B60" s="7"/>
+      <c r="B60" s="163"/>
       <c r="C60" s="7"/>
       <c r="D60" s="113">
+        <v>143638</v>
+      </c>
+      <c r="E60" s="149">
+        <f t="shared" ref="E60:E64" si="13">D60*91.91%</f>
+        <v>132017.68579999998</v>
+      </c>
+      <c r="F60" s="134">
+        <f t="shared" ref="F60:F64" si="14">D60*8.09%</f>
+        <v>11620.314200000001</v>
+      </c>
+      <c r="G60" s="109">
+        <f t="shared" ref="G60:G93" si="15">D60</f>
+        <v>143638</v>
+      </c>
+      <c r="H60" s="161">
+        <f t="shared" ref="H60:H93" si="16">E60+F60</f>
+        <v>143637.99999999997</v>
+      </c>
+      <c r="I60" s="178">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="J60" s="178">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="61" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A61" s="94" t="s">
+        <v>162</v>
+      </c>
+      <c r="B61" s="7"/>
+      <c r="C61" s="7"/>
+      <c r="D61" s="256">
         <v>129675</v>
       </c>
-      <c r="E60" s="149">
+      <c r="E61" s="149">
         <f t="shared" si="13"/>
         <v>119184.2925</v>
       </c>
-      <c r="F60" s="134">
+      <c r="F61" s="134">
         <f t="shared" si="14"/>
         <v>10490.7075</v>
       </c>
-      <c r="G60" s="109">
+      <c r="G61" s="109">
         <f t="shared" si="15"/>
         <v>129675</v>
       </c>
-      <c r="H60" s="161">
+      <c r="H61" s="161">
         <f t="shared" si="16"/>
         <v>129675</v>
       </c>
-      <c r="I60" s="178">
+      <c r="I61" s="178">
         <f t="shared" si="11"/>
         <v>0</v>
       </c>
-      <c r="J60" s="178">
+      <c r="J61" s="178">
         <f t="shared" si="12"/>
         <v>0</v>
       </c>
     </row>
-    <row r="61" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A61" s="94" t="s">
+    <row r="62" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A62" s="94" t="s">
         <v>9</v>
       </c>
-      <c r="B61" s="7" t="s">
-        <v>149</v>
-      </c>
-      <c r="C61" s="7"/>
-      <c r="D61" s="113">
+      <c r="B62" s="7" t="s">
+        <v>144</v>
+      </c>
+      <c r="C62" s="7"/>
+      <c r="D62" s="113">
         <v>74622</v>
       </c>
-      <c r="E61" s="149">
-        <f>D61*91.91%</f>
+      <c r="E62" s="149">
+        <f>D62*91.91%</f>
         <v>68585.080199999997</v>
       </c>
-      <c r="F61" s="134">
+      <c r="F62" s="134">
         <f t="shared" si="14"/>
         <v>6036.9197999999997</v>
       </c>
-      <c r="G61" s="109">
+      <c r="G62" s="109">
         <f t="shared" si="15"/>
         <v>74622</v>
       </c>
-      <c r="H61" s="161">
-        <f>E61+F61</f>
+      <c r="H62" s="161">
+        <f>E62+F62</f>
         <v>74622</v>
-      </c>
-      <c r="I61" s="178">
-        <f t="shared" si="11"/>
-        <v>0</v>
-      </c>
-      <c r="J61" s="178">
-        <f t="shared" si="12"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="62" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A62" s="94" t="s">
-        <v>11</v>
-      </c>
-      <c r="B62" s="7"/>
-      <c r="C62" s="7"/>
-      <c r="D62" s="113"/>
-      <c r="E62" s="149">
-        <f t="shared" si="13"/>
-        <v>0</v>
-      </c>
-      <c r="F62" s="134">
-        <f t="shared" si="14"/>
-        <v>0</v>
-      </c>
-      <c r="G62" s="109">
-        <f t="shared" si="15"/>
-        <v>0</v>
-      </c>
-      <c r="H62" s="161">
-        <f t="shared" si="16"/>
-        <v>0</v>
       </c>
       <c r="I62" s="178">
         <f t="shared" si="11"/>
@@ -3007,31 +3014,29 @@
       </c>
     </row>
     <row r="63" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A63" s="129" t="s">
-        <v>10</v>
-      </c>
-      <c r="B63" s="98" t="s">
-        <v>166</v>
-      </c>
-      <c r="C63" s="98"/>
-      <c r="D63" s="113">
-        <v>846331.1</v>
+      <c r="A63" s="94" t="s">
+        <v>11</v>
+      </c>
+      <c r="B63" s="7"/>
+      <c r="C63" s="7"/>
+      <c r="D63" s="256">
+        <v>614674.98</v>
       </c>
       <c r="E63" s="149">
         <f t="shared" si="13"/>
-        <v>777862.91400999995</v>
+        <v>564947.77411799994</v>
       </c>
       <c r="F63" s="134">
         <f t="shared" si="14"/>
-        <v>68468.185989999998</v>
+        <v>49727.205881999995</v>
       </c>
       <c r="G63" s="109">
         <f t="shared" si="15"/>
-        <v>846331.1</v>
+        <v>614674.98</v>
       </c>
       <c r="H63" s="161">
         <f t="shared" si="16"/>
-        <v>846331.1</v>
+        <v>614674.98</v>
       </c>
       <c r="I63" s="178">
         <f t="shared" si="11"/>
@@ -3043,26 +3048,31 @@
       </c>
     </row>
     <row r="64" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A64" s="98" t="s">
-        <v>147</v>
-      </c>
-      <c r="B64" s="179"/>
-      <c r="C64" s="180"/>
+      <c r="A64" s="129" t="s">
+        <v>10</v>
+      </c>
+      <c r="B64" s="98" t="s">
+        <v>157</v>
+      </c>
+      <c r="C64" s="98"/>
       <c r="D64" s="113">
-        <v>235500</v>
+        <v>846331.1</v>
       </c>
       <c r="E64" s="149">
-        <f t="shared" ref="E64:E76" si="17">D64</f>
-        <v>235500</v>
-      </c>
-      <c r="F64" s="134"/>
+        <f t="shared" si="13"/>
+        <v>777862.91400999995</v>
+      </c>
+      <c r="F64" s="134">
+        <f t="shared" si="14"/>
+        <v>68468.185989999998</v>
+      </c>
       <c r="G64" s="109">
         <f t="shared" si="15"/>
-        <v>235500</v>
+        <v>846331.1</v>
       </c>
       <c r="H64" s="161">
         <f t="shared" si="16"/>
-        <v>235500</v>
+        <v>846331.1</v>
       </c>
       <c r="I64" s="178">
         <f t="shared" si="11"/>
@@ -3074,29 +3084,26 @@
       </c>
     </row>
     <row r="65" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A65" s="214" t="s">
-        <v>162</v>
-      </c>
-      <c r="B65" s="215"/>
-      <c r="C65" s="216"/>
+      <c r="A65" s="98" t="s">
+        <v>143</v>
+      </c>
+      <c r="B65" s="179"/>
+      <c r="C65" s="180"/>
       <c r="D65" s="113">
-        <v>111026</v>
+        <v>235500</v>
       </c>
       <c r="E65" s="149">
-        <f>D65*91.91%</f>
-        <v>102043.99659999998</v>
-      </c>
-      <c r="F65" s="149">
-        <f>D65*8.09%</f>
-        <v>8982.0033999999996</v>
-      </c>
+        <f t="shared" ref="E65:E81" si="17">D65</f>
+        <v>235500</v>
+      </c>
+      <c r="F65" s="134"/>
       <c r="G65" s="109">
         <f t="shared" si="15"/>
-        <v>111026</v>
+        <v>235500</v>
       </c>
       <c r="H65" s="161">
-        <f>E65+F65</f>
-        <v>111025.99999999999</v>
+        <f t="shared" si="16"/>
+        <v>235500</v>
       </c>
       <c r="I65" s="178">
         <f t="shared" si="11"/>
@@ -3107,66 +3114,65 @@
         <v>0</v>
       </c>
     </row>
-    <row r="66" spans="1:10" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A66" s="214" t="s">
-        <v>157</v>
-      </c>
-      <c r="B66" s="215"/>
-      <c r="C66" s="216"/>
+    <row r="66" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A66" s="219" t="s">
+        <v>154</v>
+      </c>
+      <c r="B66" s="220"/>
+      <c r="C66" s="221"/>
       <c r="D66" s="113">
+        <v>111026</v>
+      </c>
+      <c r="E66" s="149">
+        <f>D66*91.91%</f>
+        <v>102043.99659999998</v>
+      </c>
+      <c r="F66" s="149">
+        <f>D66*8.09%</f>
+        <v>8982.0033999999996</v>
+      </c>
+      <c r="G66" s="109">
+        <f t="shared" si="15"/>
+        <v>111026</v>
+      </c>
+      <c r="H66" s="161">
+        <f>E66+F66</f>
+        <v>111025.99999999999</v>
+      </c>
+      <c r="I66" s="178">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="J66" s="178">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="67" spans="1:10" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A67" s="219" t="s">
+        <v>149</v>
+      </c>
+      <c r="B67" s="220"/>
+      <c r="C67" s="221"/>
+      <c r="D67" s="113">
         <v>104006.06</v>
       </c>
-      <c r="E66" s="149">
-        <f t="shared" ref="E66:E73" si="18">D66*91.91%</f>
+      <c r="E67" s="149">
+        <f t="shared" ref="E67:E74" si="18">D67*91.91%</f>
         <v>95591.969745999988</v>
       </c>
-      <c r="F66" s="149">
-        <f t="shared" ref="F66:F73" si="19">D66*8.09%</f>
+      <c r="F67" s="149">
+        <f t="shared" ref="F67:F74" si="19">D67*8.09%</f>
         <v>8414.0902540000006</v>
       </c>
-      <c r="G66" s="109">
-        <f>D66</f>
+      <c r="G67" s="109">
+        <f>D67</f>
         <v>104006.06</v>
       </c>
-      <c r="H66" s="161">
+      <c r="H67" s="161">
         <f t="shared" si="16"/>
         <v>104006.05999999998</v>
       </c>
-      <c r="I66" s="178">
-        <f t="shared" si="11"/>
-        <v>0</v>
-      </c>
-      <c r="J66" s="178">
-        <f t="shared" si="12"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="67" spans="1:10" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A67" s="214" t="s">
-        <v>157</v>
-      </c>
-      <c r="B67" s="215"/>
-      <c r="C67" s="216"/>
-      <c r="D67" s="113">
-        <f>104002.96</f>
-        <v>104002.96</v>
-      </c>
-      <c r="E67" s="149">
-        <f t="shared" si="18"/>
-        <v>95589.120536000002</v>
-      </c>
-      <c r="F67" s="149">
-        <f t="shared" si="19"/>
-        <v>8413.8394640000006</v>
-      </c>
-      <c r="G67" s="109">
-        <f t="shared" ref="G67:G73" si="20">D67</f>
-        <v>104002.96</v>
-      </c>
-      <c r="H67" s="161">
-        <f t="shared" si="16"/>
-        <v>104002.96</v>
-      </c>
       <c r="I67" s="178">
         <f t="shared" si="11"/>
         <v>0</v>
@@ -3177,11 +3183,11 @@
       </c>
     </row>
     <row r="68" spans="1:10" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A68" s="214" t="s">
-        <v>157</v>
-      </c>
-      <c r="B68" s="215"/>
-      <c r="C68" s="216"/>
+      <c r="A68" s="219" t="s">
+        <v>149</v>
+      </c>
+      <c r="B68" s="220"/>
+      <c r="C68" s="221"/>
       <c r="D68" s="113">
         <f>104002.96</f>
         <v>104002.96</v>
@@ -3195,7 +3201,7 @@
         <v>8413.8394640000006</v>
       </c>
       <c r="G68" s="109">
-        <f t="shared" si="20"/>
+        <f t="shared" ref="G68:G74" si="20">D68</f>
         <v>104002.96</v>
       </c>
       <c r="H68" s="161">
@@ -3212,11 +3218,11 @@
       </c>
     </row>
     <row r="69" spans="1:10" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A69" s="214" t="s">
-        <v>157</v>
-      </c>
-      <c r="B69" s="215"/>
-      <c r="C69" s="216"/>
+      <c r="A69" s="219" t="s">
+        <v>149</v>
+      </c>
+      <c r="B69" s="220"/>
+      <c r="C69" s="221"/>
       <c r="D69" s="113">
         <f>104002.96</f>
         <v>104002.96</v>
@@ -3247,29 +3253,30 @@
       </c>
     </row>
     <row r="70" spans="1:10" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A70" s="228" t="s">
-        <v>156</v>
-      </c>
-      <c r="B70" s="229"/>
-      <c r="C70" s="230"/>
+      <c r="A70" s="219" t="s">
+        <v>149</v>
+      </c>
+      <c r="B70" s="220"/>
+      <c r="C70" s="221"/>
       <c r="D70" s="113">
-        <v>100419.01</v>
+        <f>104002.96</f>
+        <v>104002.96</v>
       </c>
       <c r="E70" s="149">
         <f t="shared" si="18"/>
-        <v>92295.112090999988</v>
+        <v>95589.120536000002</v>
       </c>
       <c r="F70" s="149">
         <f t="shared" si="19"/>
-        <v>8123.8979089999993</v>
+        <v>8413.8394640000006</v>
       </c>
       <c r="G70" s="109">
         <f t="shared" si="20"/>
-        <v>100419.01</v>
+        <v>104002.96</v>
       </c>
       <c r="H70" s="161">
         <f t="shared" si="16"/>
-        <v>100419.00999999998</v>
+        <v>104002.96</v>
       </c>
       <c r="I70" s="178">
         <f t="shared" si="11"/>
@@ -3281,29 +3288,29 @@
       </c>
     </row>
     <row r="71" spans="1:10" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A71" s="228" t="s">
-        <v>156</v>
-      </c>
-      <c r="B71" s="229"/>
-      <c r="C71" s="230"/>
+      <c r="A71" s="202" t="s">
+        <v>148</v>
+      </c>
+      <c r="B71" s="203"/>
+      <c r="C71" s="204"/>
       <c r="D71" s="113">
-        <v>97003.05</v>
+        <v>100419.01</v>
       </c>
       <c r="E71" s="149">
         <f t="shared" si="18"/>
-        <v>89155.503254999989</v>
+        <v>92295.112090999988</v>
       </c>
       <c r="F71" s="149">
         <f t="shared" si="19"/>
-        <v>7847.5467450000006</v>
+        <v>8123.8979089999993</v>
       </c>
       <c r="G71" s="109">
         <f t="shared" si="20"/>
-        <v>97003.05</v>
+        <v>100419.01</v>
       </c>
       <c r="H71" s="161">
         <f t="shared" si="16"/>
-        <v>97003.049999999988</v>
+        <v>100419.00999999998</v>
       </c>
       <c r="I71" s="178">
         <f t="shared" si="11"/>
@@ -3315,29 +3322,29 @@
       </c>
     </row>
     <row r="72" spans="1:10" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A72" s="228" t="s">
-        <v>155</v>
-      </c>
-      <c r="B72" s="229"/>
-      <c r="C72" s="230"/>
+      <c r="A72" s="202" t="s">
+        <v>148</v>
+      </c>
+      <c r="B72" s="203"/>
+      <c r="C72" s="204"/>
       <c r="D72" s="113">
-        <v>98393.96</v>
+        <v>97003.05</v>
       </c>
       <c r="E72" s="149">
         <f t="shared" si="18"/>
-        <v>90433.888636000003</v>
+        <v>89155.503254999989</v>
       </c>
       <c r="F72" s="149">
         <f t="shared" si="19"/>
-        <v>7960.0713640000004</v>
+        <v>7847.5467450000006</v>
       </c>
       <c r="G72" s="109">
         <f t="shared" si="20"/>
-        <v>98393.96</v>
+        <v>97003.05</v>
       </c>
       <c r="H72" s="161">
         <f t="shared" si="16"/>
-        <v>98393.96</v>
+        <v>97003.049999999988</v>
       </c>
       <c r="I72" s="178">
         <f t="shared" si="11"/>
@@ -3349,29 +3356,29 @@
       </c>
     </row>
     <row r="73" spans="1:10" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A73" s="197" t="s">
-        <v>165</v>
-      </c>
-      <c r="B73" s="195"/>
-      <c r="C73" s="196"/>
+      <c r="A73" s="202" t="s">
+        <v>147</v>
+      </c>
+      <c r="B73" s="203"/>
+      <c r="C73" s="204"/>
       <c r="D73" s="113">
-        <v>99259.05</v>
+        <v>98393.96</v>
       </c>
       <c r="E73" s="149">
         <f t="shared" si="18"/>
-        <v>91228.99285499999</v>
+        <v>90433.888636000003</v>
       </c>
       <c r="F73" s="149">
         <f t="shared" si="19"/>
-        <v>8030.0571449999998</v>
+        <v>7960.0713640000004</v>
       </c>
       <c r="G73" s="109">
         <f t="shared" si="20"/>
-        <v>99259.05</v>
+        <v>98393.96</v>
       </c>
       <c r="H73" s="161">
         <f t="shared" si="16"/>
-        <v>99259.049999999988</v>
+        <v>98393.96</v>
       </c>
       <c r="I73" s="178">
         <f t="shared" si="11"/>
@@ -3382,58 +3389,61 @@
         <v>0</v>
       </c>
     </row>
-    <row r="74" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A74" s="225" t="s">
-        <v>145</v>
-      </c>
-      <c r="B74" s="226"/>
-      <c r="C74" s="227"/>
+    <row r="74" spans="1:10" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A74" s="197" t="s">
+        <v>156</v>
+      </c>
+      <c r="B74" s="195"/>
+      <c r="C74" s="196"/>
       <c r="D74" s="113">
+        <v>99259.05</v>
+      </c>
+      <c r="E74" s="149">
+        <f t="shared" si="18"/>
+        <v>91228.99285499999</v>
+      </c>
+      <c r="F74" s="149">
+        <f t="shared" si="19"/>
+        <v>8030.0571449999998</v>
+      </c>
+      <c r="G74" s="109">
+        <f t="shared" si="20"/>
+        <v>99259.05</v>
+      </c>
+      <c r="H74" s="161">
+        <f t="shared" si="16"/>
+        <v>99259.049999999988</v>
+      </c>
+      <c r="I74" s="178">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="J74" s="178">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="75" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A75" s="230" t="s">
+        <v>170</v>
+      </c>
+      <c r="B75" s="231"/>
+      <c r="C75" s="232"/>
+      <c r="D75" s="256">
         <v>66000</v>
       </c>
-      <c r="E74" s="149">
+      <c r="E75" s="149">
         <f t="shared" si="17"/>
         <v>66000</v>
-      </c>
-      <c r="F74" s="134"/>
-      <c r="G74" s="109">
-        <f t="shared" si="15"/>
-        <v>66000</v>
-      </c>
-      <c r="H74" s="161">
-        <f t="shared" si="16"/>
-        <v>66000</v>
-      </c>
-      <c r="I74" s="178">
-        <f t="shared" si="11"/>
-        <v>0</v>
-      </c>
-      <c r="J74" s="178">
-        <f t="shared" si="12"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="75" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A75" s="231" t="s">
-        <v>151</v>
-      </c>
-      <c r="B75" s="232"/>
-      <c r="C75" s="233"/>
-      <c r="D75" s="113">
-        <v>218400</v>
-      </c>
-      <c r="E75" s="149">
-        <f t="shared" si="17"/>
-        <v>218400</v>
       </c>
       <c r="F75" s="134"/>
       <c r="G75" s="109">
         <f t="shared" si="15"/>
-        <v>218400</v>
+        <v>66000</v>
       </c>
       <c r="H75" s="161">
         <f t="shared" si="16"/>
-        <v>218400</v>
+        <v>66000</v>
       </c>
       <c r="I75" s="178">
         <f t="shared" si="11"/>
@@ -3445,26 +3455,26 @@
       </c>
     </row>
     <row r="76" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A76" s="193" t="s">
-        <v>148</v>
-      </c>
-      <c r="B76" s="194"/>
-      <c r="C76" s="189"/>
+      <c r="A76" s="233" t="s">
+        <v>145</v>
+      </c>
+      <c r="B76" s="234"/>
+      <c r="C76" s="235"/>
       <c r="D76" s="113">
-        <v>35000</v>
+        <v>218400</v>
       </c>
       <c r="E76" s="149">
         <f t="shared" si="17"/>
-        <v>35000</v>
+        <v>218400</v>
       </c>
       <c r="F76" s="134"/>
       <c r="G76" s="109">
         <f t="shared" si="15"/>
-        <v>35000</v>
+        <v>218400</v>
       </c>
       <c r="H76" s="161">
         <f t="shared" si="16"/>
-        <v>35000</v>
+        <v>218400</v>
       </c>
       <c r="I76" s="178">
         <f t="shared" si="11"/>
@@ -3476,62 +3486,54 @@
       </c>
     </row>
     <row r="77" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A77" s="7" t="s">
-        <v>120</v>
-      </c>
-      <c r="B77" s="7" t="s">
+      <c r="A77" s="259" t="s">
         <v>173</v>
       </c>
+      <c r="B77" s="7"/>
       <c r="C77" s="7"/>
-      <c r="D77" s="113">
-        <v>79895</v>
+      <c r="D77" s="256">
+        <v>315000</v>
       </c>
       <c r="E77" s="149">
-        <f t="shared" ref="E77:E84" si="21">D77</f>
-        <v>79895</v>
-      </c>
-      <c r="F77" s="7"/>
+        <f t="shared" si="17"/>
+        <v>315000</v>
+      </c>
+      <c r="F77" s="134"/>
       <c r="G77" s="109">
         <f t="shared" si="15"/>
-        <v>79895</v>
+        <v>315000</v>
       </c>
       <c r="H77" s="161">
         <f t="shared" si="16"/>
-        <v>79895</v>
+        <v>315000</v>
       </c>
       <c r="I77" s="178">
         <f t="shared" si="11"/>
         <v>0</v>
       </c>
-      <c r="J77" s="178">
-        <f t="shared" si="12"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="78" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A78" s="94" t="s">
-        <v>139</v>
-      </c>
-      <c r="B78" s="7"/>
-      <c r="C78" s="7"/>
-      <c r="D78" s="113">
-        <v>6530.7</v>
+      <c r="J77" s="178"/>
+    </row>
+    <row r="78" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A78" s="193" t="s">
+        <v>169</v>
+      </c>
+      <c r="B78" s="194"/>
+      <c r="C78" s="189"/>
+      <c r="D78" s="256">
+        <v>35000</v>
       </c>
       <c r="E78" s="149">
-        <f t="shared" ref="E78:E82" si="22">D78*91.91%</f>
-        <v>6002.3663699999997</v>
-      </c>
-      <c r="F78" s="134">
-        <f t="shared" ref="F78:F82" si="23">D78*8.09%</f>
-        <v>528.33362999999997</v>
-      </c>
+        <f t="shared" si="17"/>
+        <v>35000</v>
+      </c>
+      <c r="F78" s="134"/>
       <c r="G78" s="109">
         <f t="shared" si="15"/>
-        <v>6530.7</v>
+        <v>35000</v>
       </c>
       <c r="H78" s="161">
         <f t="shared" si="16"/>
-        <v>6530.7</v>
+        <v>35000</v>
       </c>
       <c r="I78" s="178">
         <f t="shared" si="11"/>
@@ -3542,95 +3544,83 @@
         <v>0</v>
       </c>
     </row>
-    <row r="79" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A79" s="94" t="s">
-        <v>150</v>
-      </c>
-      <c r="B79" s="7"/>
+    <row r="79" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A79" s="258" t="s">
+        <v>174</v>
+      </c>
+      <c r="B79" s="114"/>
       <c r="C79" s="7"/>
-      <c r="D79" s="113">
-        <v>220000</v>
+      <c r="D79" s="256">
+        <v>143416.32999999999</v>
       </c>
       <c r="E79" s="149">
-        <f t="shared" si="22"/>
-        <v>202201.99999999997</v>
-      </c>
-      <c r="F79" s="134">
-        <f t="shared" si="23"/>
-        <v>17798</v>
-      </c>
+        <f t="shared" si="17"/>
+        <v>143416.32999999999</v>
+      </c>
+      <c r="F79" s="134"/>
       <c r="G79" s="109">
         <f t="shared" si="15"/>
-        <v>220000</v>
+        <v>143416.32999999999</v>
       </c>
       <c r="H79" s="161">
         <f t="shared" si="16"/>
-        <v>219999.99999999997</v>
+        <v>143416.32999999999</v>
       </c>
       <c r="I79" s="178">
-        <f>H79-D79</f>
-        <v>0</v>
-      </c>
-      <c r="J79" s="178">
-        <f t="shared" si="12"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="80" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A80" s="94" t="s">
-        <v>154</v>
-      </c>
-      <c r="B80" s="7"/>
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="J79" s="178"/>
+    </row>
+    <row r="80" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A80" s="7" t="s">
+        <v>175</v>
+      </c>
+      <c r="B80" s="114"/>
       <c r="C80" s="7"/>
-      <c r="D80" s="113">
-        <v>150000</v>
+      <c r="D80" s="256">
+        <v>12100</v>
       </c>
       <c r="E80" s="149">
-        <f t="shared" si="22"/>
-        <v>137865</v>
-      </c>
-      <c r="F80" s="134">
-        <f t="shared" si="23"/>
-        <v>12135</v>
-      </c>
+        <f t="shared" si="17"/>
+        <v>12100</v>
+      </c>
+      <c r="F80" s="134"/>
       <c r="G80" s="109">
         <f t="shared" si="15"/>
-        <v>150000</v>
+        <v>12100</v>
       </c>
       <c r="H80" s="161">
         <f t="shared" si="16"/>
-        <v>150000</v>
+        <v>12100</v>
       </c>
       <c r="I80" s="178">
         <f t="shared" si="11"/>
         <v>0</v>
       </c>
-      <c r="J80" s="178">
-        <f t="shared" si="12"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="81" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A81" s="7" t="s">
-        <v>146</v>
-      </c>
-      <c r="B81" s="7"/>
+      <c r="J80" s="178"/>
+    </row>
+    <row r="81" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A81" s="257" t="s">
+        <v>176</v>
+      </c>
+      <c r="B81" s="114"/>
       <c r="C81" s="7"/>
-      <c r="D81" s="113">
-        <v>120000</v>
+      <c r="D81" s="256">
+        <v>4200</v>
       </c>
       <c r="E81" s="149">
-        <f t="shared" si="21"/>
-        <v>120000</v>
+        <f t="shared" si="17"/>
+        <v>4200</v>
       </c>
       <c r="F81" s="7"/>
       <c r="G81" s="109">
         <f t="shared" si="15"/>
-        <v>120000</v>
+        <v>4200</v>
       </c>
       <c r="H81" s="161">
         <f t="shared" si="16"/>
-        <v>120000</v>
+        <v>4200</v>
       </c>
       <c r="I81" s="178">
         <f t="shared" si="11"/>
@@ -3642,29 +3632,29 @@
       </c>
     </row>
     <row r="82" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A82" s="94" t="s">
-        <v>152</v>
-      </c>
-      <c r="B82" s="114"/>
+      <c r="A82" s="255" t="s">
+        <v>167</v>
+      </c>
+      <c r="B82" s="7"/>
       <c r="C82" s="7"/>
-      <c r="D82" s="113">
-        <v>245000</v>
+      <c r="D82" s="256">
+        <v>736429.26</v>
       </c>
       <c r="E82" s="149">
-        <f t="shared" si="22"/>
-        <v>225179.49999999997</v>
+        <f t="shared" ref="E82:E89" si="21">D82*91.91%</f>
+        <v>676852.13286599994</v>
       </c>
       <c r="F82" s="134">
-        <f t="shared" si="23"/>
-        <v>19820.5</v>
+        <f t="shared" ref="F82:F90" si="22">D82*8.09%</f>
+        <v>59577.127134000002</v>
       </c>
       <c r="G82" s="109">
         <f t="shared" si="15"/>
-        <v>245000</v>
+        <v>736429.26</v>
       </c>
       <c r="H82" s="161">
         <f t="shared" si="16"/>
-        <v>244999.99999999997</v>
+        <v>736429.25999999989</v>
       </c>
       <c r="I82" s="178">
         <f t="shared" si="11"/>
@@ -3676,26 +3666,29 @@
       </c>
     </row>
     <row r="83" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A83" s="7" t="s">
-        <v>142</v>
-      </c>
-      <c r="B83" s="114"/>
+      <c r="A83" s="255" t="s">
+        <v>167</v>
+      </c>
+      <c r="B83" s="7"/>
       <c r="C83" s="7"/>
-      <c r="D83" s="113">
-        <v>120000</v>
+      <c r="D83" s="256">
+        <v>232510.18</v>
       </c>
       <c r="E83" s="149">
         <f t="shared" si="21"/>
-        <v>120000</v>
-      </c>
-      <c r="F83" s="7"/>
+        <v>213700.10643799999</v>
+      </c>
+      <c r="F83" s="134">
+        <f t="shared" si="22"/>
+        <v>18810.073561999998</v>
+      </c>
       <c r="G83" s="109">
         <f t="shared" si="15"/>
-        <v>120000</v>
+        <v>232510.18</v>
       </c>
       <c r="H83" s="161">
         <f t="shared" si="16"/>
-        <v>120000</v>
+        <v>232510.18</v>
       </c>
       <c r="I83" s="178">
         <f t="shared" si="11"/>
@@ -3707,26 +3700,29 @@
       </c>
     </row>
     <row r="84" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A84" s="7" t="s">
-        <v>164</v>
-      </c>
-      <c r="B84" s="114"/>
+      <c r="A84" s="255" t="s">
+        <v>167</v>
+      </c>
+      <c r="B84" s="7"/>
       <c r="C84" s="7"/>
-      <c r="D84" s="113">
-        <v>480000</v>
+      <c r="D84" s="256">
+        <v>357622.29</v>
       </c>
       <c r="E84" s="149">
         <f t="shared" si="21"/>
-        <v>480000</v>
-      </c>
-      <c r="F84" s="7"/>
+        <v>328690.64673899993</v>
+      </c>
+      <c r="F84" s="134">
+        <f t="shared" si="22"/>
+        <v>28931.643260999997</v>
+      </c>
       <c r="G84" s="109">
         <f t="shared" si="15"/>
-        <v>480000</v>
+        <v>357622.29</v>
       </c>
       <c r="H84" s="161">
         <f t="shared" si="16"/>
-        <v>480000</v>
+        <v>357622.28999999992</v>
       </c>
       <c r="I84" s="178">
         <f t="shared" si="11"/>
@@ -3738,220 +3734,352 @@
       </c>
     </row>
     <row r="85" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A85" s="94" t="s">
+      <c r="A85" s="255" t="s">
         <v>167</v>
       </c>
-      <c r="B85" s="114"/>
+      <c r="B85" s="7"/>
       <c r="C85" s="7"/>
-      <c r="D85" s="113">
-        <v>250000</v>
+      <c r="D85" s="256">
+        <v>358487.12</v>
       </c>
       <c r="E85" s="149">
-        <f t="shared" ref="E85:E86" si="24">D85*91.91%</f>
-        <v>229774.99999999997</v>
+        <f t="shared" si="21"/>
+        <v>329485.51199199999</v>
       </c>
       <c r="F85" s="134">
-        <f t="shared" ref="F85:F86" si="25">D85*8.09%</f>
-        <v>20225</v>
+        <f t="shared" si="22"/>
+        <v>29001.608007999999</v>
       </c>
       <c r="G85" s="109">
         <f t="shared" si="15"/>
-        <v>250000</v>
-      </c>
-      <c r="H85" s="161"/>
-      <c r="I85" s="178"/>
+        <v>358487.12</v>
+      </c>
+      <c r="H85" s="161">
+        <f t="shared" si="16"/>
+        <v>358487.12</v>
+      </c>
+      <c r="I85" s="178">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
       <c r="J85" s="178">
         <f t="shared" si="12"/>
         <v>0</v>
       </c>
     </row>
     <row r="86" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A86" s="129" t="s">
-        <v>158</v>
-      </c>
-      <c r="B86" s="114"/>
-      <c r="C86" s="162"/>
-      <c r="D86" s="113">
+      <c r="A86" s="255" t="s">
+        <v>167</v>
+      </c>
+      <c r="B86" s="7"/>
+      <c r="C86" s="7"/>
+      <c r="D86" s="256">
+        <v>186859.86</v>
+      </c>
+      <c r="E86" s="149">
+        <f t="shared" si="21"/>
+        <v>171742.89732599998</v>
+      </c>
+      <c r="F86" s="134">
+        <f t="shared" si="22"/>
+        <v>15116.962673999999</v>
+      </c>
+      <c r="G86" s="109">
+        <f t="shared" si="15"/>
+        <v>186859.86</v>
+      </c>
+      <c r="H86" s="161">
+        <f t="shared" si="16"/>
+        <v>186859.86</v>
+      </c>
+      <c r="I86" s="178">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="J86" s="178">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="87" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A87" s="257" t="s">
+        <v>171</v>
+      </c>
+      <c r="B87" s="7"/>
+      <c r="C87" s="7"/>
+      <c r="D87" s="256">
+        <v>36300</v>
+      </c>
+      <c r="E87" s="149">
+        <f t="shared" si="21"/>
+        <v>33363.329999999994</v>
+      </c>
+      <c r="F87" s="134">
+        <f t="shared" si="22"/>
+        <v>2936.67</v>
+      </c>
+      <c r="G87" s="109">
+        <f t="shared" si="15"/>
+        <v>36300</v>
+      </c>
+      <c r="H87" s="161">
+        <f t="shared" si="16"/>
+        <v>36299.999999999993</v>
+      </c>
+      <c r="I87" s="178">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="J87" s="178">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="88" spans="1:10" ht="41.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A88" s="230" t="s">
+        <v>172</v>
+      </c>
+      <c r="B88" s="231"/>
+      <c r="C88" s="232"/>
+      <c r="D88" s="256">
+        <v>430000</v>
+      </c>
+      <c r="E88" s="149">
+        <f t="shared" ref="E81:E91" si="23">D88</f>
+        <v>430000</v>
+      </c>
+      <c r="F88" s="7"/>
+      <c r="G88" s="109">
+        <f t="shared" si="15"/>
+        <v>430000</v>
+      </c>
+      <c r="H88" s="161">
+        <f t="shared" si="16"/>
+        <v>430000</v>
+      </c>
+      <c r="I88" s="178">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="J88" s="178">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="89" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A89" s="7" t="s">
+        <v>120</v>
+      </c>
+      <c r="B89" s="7" t="s">
+        <v>163</v>
+      </c>
+      <c r="C89" s="7"/>
+      <c r="D89" s="113">
+        <v>79895</v>
+      </c>
+      <c r="E89" s="149">
+        <f t="shared" si="21"/>
+        <v>73431.494499999986</v>
+      </c>
+      <c r="F89" s="134">
+        <f t="shared" si="22"/>
+        <v>6463.5055000000002</v>
+      </c>
+      <c r="G89" s="109">
+        <f t="shared" si="15"/>
+        <v>79895</v>
+      </c>
+      <c r="H89" s="161">
+        <f t="shared" si="16"/>
+        <v>79894.999999999985</v>
+      </c>
+      <c r="I89" s="178">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="J89" s="178">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="90" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A90" s="258" t="s">
+        <v>177</v>
+      </c>
+      <c r="B90" s="114"/>
+      <c r="C90" s="7"/>
+      <c r="D90" s="256">
+        <v>180000</v>
+      </c>
+      <c r="E90" s="149">
+        <f t="shared" si="23"/>
+        <v>180000</v>
+      </c>
+      <c r="F90" s="7">
+        <f t="shared" si="22"/>
+        <v>14562</v>
+      </c>
+      <c r="G90" s="109">
+        <f t="shared" si="15"/>
+        <v>180000</v>
+      </c>
+      <c r="H90" s="161">
+        <f t="shared" si="16"/>
+        <v>194562</v>
+      </c>
+      <c r="I90" s="178">
+        <f t="shared" si="11"/>
+        <v>14562</v>
+      </c>
+      <c r="J90" s="178">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="91" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A91" s="7"/>
+      <c r="B91" s="114"/>
+      <c r="C91" s="7"/>
+      <c r="D91" s="256"/>
+      <c r="E91" s="149">
+        <f t="shared" si="23"/>
+        <v>0</v>
+      </c>
+      <c r="F91" s="7"/>
+      <c r="G91" s="109">
+        <f t="shared" si="15"/>
+        <v>0</v>
+      </c>
+      <c r="H91" s="161">
+        <f t="shared" si="16"/>
+        <v>0</v>
+      </c>
+      <c r="I91" s="178">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="J91" s="178">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="92" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A92" s="94"/>
+      <c r="B92" s="114"/>
+      <c r="C92" s="7"/>
+      <c r="D92" s="256"/>
+      <c r="E92" s="149">
+        <f t="shared" ref="E92:E93" si="24">D92*91.91%</f>
+        <v>0</v>
+      </c>
+      <c r="F92" s="134">
+        <f t="shared" ref="F92:F93" si="25">D92*8.09%</f>
+        <v>0</v>
+      </c>
+      <c r="G92" s="109">
+        <f t="shared" si="15"/>
+        <v>0</v>
+      </c>
+      <c r="H92" s="161"/>
+      <c r="I92" s="178">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="J92" s="178">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="93" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A93" s="129" t="s">
+        <v>150</v>
+      </c>
+      <c r="B93" s="114"/>
+      <c r="C93" s="162"/>
+      <c r="D93" s="113">
         <v>50000</v>
       </c>
-      <c r="E86" s="149">
+      <c r="E93" s="149">
         <f t="shared" si="24"/>
         <v>45954.999999999993</v>
       </c>
-      <c r="F86" s="134">
+      <c r="F93" s="134">
         <f t="shared" si="25"/>
         <v>4045</v>
       </c>
-      <c r="G86" s="109">
+      <c r="G93" s="109">
         <f t="shared" si="15"/>
         <v>50000</v>
       </c>
-      <c r="H86" s="161">
+      <c r="H93" s="161">
         <f t="shared" si="16"/>
         <v>49999.999999999993</v>
       </c>
-      <c r="I86" s="178">
+      <c r="I93" s="178">
         <f t="shared" si="11"/>
         <v>0</v>
       </c>
-      <c r="J86" s="178">
+      <c r="J93" s="178">
         <f t="shared" si="12"/>
         <v>0</v>
       </c>
     </row>
-    <row r="87" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A87" s="155"/>
-      <c r="B87" s="156"/>
-      <c r="C87" s="156"/>
-      <c r="D87" s="166"/>
-      <c r="E87" s="149"/>
-      <c r="F87" s="134"/>
-      <c r="G87" s="109"/>
-      <c r="H87" s="161"/>
-      <c r="I87" t="str">
-        <f>IF(G87=H87, "", "Error")</f>
+    <row r="94" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A94" s="155"/>
+      <c r="B94" s="156"/>
+      <c r="C94" s="156"/>
+      <c r="D94" s="166"/>
+      <c r="E94" s="149"/>
+      <c r="F94" s="134"/>
+      <c r="G94" s="109"/>
+      <c r="H94" s="161"/>
+      <c r="I94" t="str">
+        <f>IF(G94=H94, "", "Error")</f>
         <v/>
       </c>
     </row>
-    <row r="88" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A88" s="96" t="s">
+    <row r="95" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A95" s="96" t="s">
         <v>12</v>
       </c>
-      <c r="B88" s="96"/>
-      <c r="C88" s="96"/>
-      <c r="D88" s="108">
-        <f>SUM(D57:D87)</f>
-        <v>5422707.8099999996</v>
-      </c>
-      <c r="E88" s="108">
-        <f>SUM(E57:E87)</f>
-        <v>5176940.6636709999</v>
-      </c>
-      <c r="F88" s="108">
-        <f>SUM(F57:F87)</f>
-        <v>245767.14632900001</v>
-      </c>
-      <c r="G88" s="109">
-        <f>E88+F88</f>
-        <v>5422707.8099999996</v>
-      </c>
-      <c r="H88" s="150" t="str">
-        <f>IF(D88=G88, "", "Error")</f>
-        <v/>
-      </c>
-      <c r="I88" s="178">
-        <f>D88-G88</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="89" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A89" s="7"/>
-      <c r="B89" s="7"/>
-      <c r="C89" s="7"/>
-      <c r="D89" s="185"/>
-      <c r="E89" s="115"/>
-      <c r="F89" s="7"/>
-      <c r="H89" s="150"/>
-    </row>
-    <row r="90" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A90" s="7"/>
-      <c r="B90" s="7"/>
-      <c r="C90" s="7"/>
-      <c r="D90" s="185"/>
-      <c r="E90" s="114"/>
-      <c r="F90" s="7"/>
-      <c r="H90" s="150"/>
-    </row>
-    <row r="91" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A91" s="7"/>
-      <c r="B91" s="7"/>
-      <c r="C91" s="7"/>
-      <c r="D91" s="185"/>
-      <c r="E91" s="114"/>
-      <c r="F91" s="7"/>
-      <c r="H91" s="150"/>
-    </row>
-    <row r="92" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A92" s="94" t="s">
-        <v>161</v>
-      </c>
-      <c r="B92" s="98"/>
-      <c r="C92" s="7"/>
-      <c r="D92" s="113"/>
-      <c r="E92" s="149">
-        <f>D92*91.91%</f>
-        <v>0</v>
-      </c>
-      <c r="F92" s="134">
-        <f>D92*8.09%</f>
-        <v>0</v>
-      </c>
-      <c r="G92" s="160"/>
-      <c r="H92" s="150"/>
-    </row>
-    <row r="93" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A93" s="7"/>
-      <c r="B93" s="7"/>
-      <c r="C93" s="7"/>
-      <c r="D93" s="113"/>
-      <c r="E93" s="164">
-        <f>D93</f>
-        <v>0</v>
-      </c>
-      <c r="F93" s="7"/>
-      <c r="H93" s="150"/>
-      <c r="I93" s="109"/>
-    </row>
-    <row r="94" spans="1:10" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A94" s="95" t="s">
-        <v>17</v>
-      </c>
-      <c r="B94" s="95"/>
-      <c r="C94" s="95"/>
-      <c r="D94" s="107">
-        <f>SUM(D92:D93)</f>
-        <v>0</v>
-      </c>
-      <c r="E94" s="107">
-        <f>SUM(E92:E93)</f>
-        <v>0</v>
-      </c>
-      <c r="F94" s="107">
-        <f>SUM(F92:F93)</f>
-        <v>0</v>
-      </c>
-      <c r="G94" s="109">
-        <f>E94+F94</f>
-        <v>0</v>
-      </c>
-      <c r="H94" s="150" t="str">
-        <f>IF(D94=G94, "", "Error")</f>
-        <v/>
-      </c>
-      <c r="J94" s="109"/>
-    </row>
-    <row r="95" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A95" s="7"/>
-      <c r="B95" s="7"/>
-      <c r="C95" s="7"/>
-      <c r="D95" s="185"/>
-      <c r="E95" s="115"/>
-      <c r="F95" s="7"/>
-      <c r="H95" s="150"/>
+      <c r="B95" s="96"/>
+      <c r="C95" s="96"/>
+      <c r="D95" s="108">
+        <f>SUM(D57:D94)</f>
+        <v>8463777.129999999</v>
+      </c>
+      <c r="E95" s="108">
+        <f>SUM(E57:E94)</f>
+        <v>8077952.02128</v>
+      </c>
+      <c r="F95" s="108">
+        <f>SUM(F57:F94)</f>
+        <v>400387.10871999996</v>
+      </c>
+      <c r="G95" s="109">
+        <f>E95+F95</f>
+        <v>8478339.1300000008</v>
+      </c>
+      <c r="H95" s="150" t="str">
+        <f>IF(D95=G95, "", "Error")</f>
+        <v>Error</v>
+      </c>
+      <c r="I95" s="178">
+        <f>D95-G95</f>
+        <v>-14562.000000001863</v>
+      </c>
     </row>
     <row r="96" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A96" s="7"/>
       <c r="B96" s="7"/>
       <c r="C96" s="7"/>
       <c r="D96" s="185"/>
-      <c r="E96" s="114"/>
+      <c r="E96" s="115"/>
       <c r="F96" s="7"/>
       <c r="H96" s="150"/>
     </row>
-    <row r="97" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A97" s="94" t="s">
-        <v>13</v>
-      </c>
+    <row r="97" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A97" s="7"/>
       <c r="B97" s="7"/>
       <c r="C97" s="7"/>
       <c r="D97" s="185"/>
@@ -3959,78 +4087,70 @@
       <c r="F97" s="7"/>
       <c r="H97" s="150"/>
     </row>
-    <row r="98" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A98" s="94" t="s">
-        <v>14</v>
-      </c>
-      <c r="B98" s="7" t="s">
-        <v>117</v>
-      </c>
+    <row r="98" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A98" s="7"/>
+      <c r="B98" s="7"/>
       <c r="C98" s="7"/>
-      <c r="D98" s="113">
-        <v>222264.92</v>
-      </c>
-      <c r="E98" s="149">
-        <f>D98*91.91%</f>
-        <v>204283.68797199999</v>
-      </c>
-      <c r="F98" s="134">
-        <f>D98*8.09%</f>
-        <v>17981.232028000002</v>
-      </c>
+      <c r="D98" s="185"/>
+      <c r="E98" s="114"/>
+      <c r="F98" s="7"/>
       <c r="H98" s="150"/>
     </row>
     <row r="99" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A99" s="94" t="s">
-        <v>108</v>
-      </c>
-      <c r="B99" s="7"/>
+        <v>153</v>
+      </c>
+      <c r="B99" s="98"/>
       <c r="C99" s="7"/>
-      <c r="D99" s="113">
-        <v>28000</v>
+      <c r="D99" s="256">
+        <f>67780+35700</f>
+        <v>103480</v>
       </c>
       <c r="E99" s="149">
         <f>D99*91.91%</f>
-        <v>25734.799999999999</v>
+        <v>95108.467999999993</v>
       </c>
       <c r="F99" s="134">
         <f>D99*8.09%</f>
-        <v>2265.1999999999998</v>
-      </c>
+        <v>8371.5319999999992</v>
+      </c>
+      <c r="G99" s="160"/>
       <c r="H99" s="150"/>
-      <c r="J99" s="113"/>
     </row>
     <row r="100" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A100" s="7"/>
       <c r="B100" s="7"/>
       <c r="C100" s="7"/>
-      <c r="D100" s="185"/>
-      <c r="E100" s="116"/>
+      <c r="D100" s="113"/>
+      <c r="E100" s="164">
+        <f>D100</f>
+        <v>0</v>
+      </c>
       <c r="F100" s="7"/>
       <c r="H100" s="150"/>
-      <c r="J100" s="109"/>
-    </row>
-    <row r="101" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="I100" s="109"/>
+    </row>
+    <row r="101" spans="1:10" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A101" s="95" t="s">
-        <v>101</v>
+        <v>17</v>
       </c>
       <c r="B101" s="95"/>
       <c r="C101" s="95"/>
       <c r="D101" s="107">
-        <f>SUM(D98:D100)</f>
-        <v>250264.92</v>
+        <f>SUM(D99:D100)</f>
+        <v>103480</v>
       </c>
       <c r="E101" s="107">
-        <f>SUM(E98:E100)</f>
-        <v>230018.48797199997</v>
+        <f>SUM(E99:E100)</f>
+        <v>95108.467999999993</v>
       </c>
       <c r="F101" s="107">
-        <f>SUM(F98:F100)</f>
-        <v>20246.432028000003</v>
+        <f>SUM(F99:F100)</f>
+        <v>8371.5319999999992</v>
       </c>
       <c r="G101" s="109">
         <f>E101+F101</f>
-        <v>250264.91999999998</v>
+        <v>103480</v>
       </c>
       <c r="H101" s="150" t="str">
         <f>IF(D101=G101, "", "Error")</f>
@@ -4038,555 +4158,664 @@
       </c>
       <c r="J101" s="109"/>
     </row>
-    <row r="102" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A102" s="7"/>
       <c r="B102" s="7"/>
       <c r="C102" s="7"/>
-      <c r="D102" s="113"/>
-      <c r="E102" s="117"/>
+      <c r="D102" s="185"/>
+      <c r="E102" s="115"/>
       <c r="F102" s="7"/>
       <c r="H102" s="150"/>
     </row>
-    <row r="103" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A103" s="94" t="s">
-        <v>102</v>
-      </c>
+    <row r="103" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A103" s="7"/>
       <c r="B103" s="7"/>
       <c r="C103" s="7"/>
-      <c r="D103" s="113">
-        <v>100104.56</v>
-      </c>
-      <c r="E103" s="149">
-        <f>D103*91.91%</f>
-        <v>92006.101095999984</v>
-      </c>
-      <c r="F103" s="134">
-        <f>D103*8.09%</f>
-        <v>8098.4589040000001</v>
-      </c>
+      <c r="D103" s="185"/>
+      <c r="E103" s="114"/>
+      <c r="F103" s="7"/>
       <c r="H103" s="150"/>
     </row>
     <row r="104" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A104" s="94" t="s">
+        <v>13</v>
+      </c>
+      <c r="B104" s="7"/>
+      <c r="C104" s="7"/>
+      <c r="D104" s="185"/>
+      <c r="E104" s="114"/>
+      <c r="F104" s="7"/>
+      <c r="H104" s="150"/>
+    </row>
+    <row r="105" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A105" s="94" t="s">
+        <v>14</v>
+      </c>
+      <c r="B105" s="7" t="s">
+        <v>117</v>
+      </c>
+      <c r="C105" s="7"/>
+      <c r="D105" s="113">
+        <v>222264.92</v>
+      </c>
+      <c r="E105" s="149">
+        <f>D105*91.91%</f>
+        <v>204283.68797199999</v>
+      </c>
+      <c r="F105" s="134">
+        <f>D105*8.09%</f>
+        <v>17981.232028000002</v>
+      </c>
+      <c r="H105" s="150"/>
+    </row>
+    <row r="106" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A106" s="94" t="s">
+        <v>108</v>
+      </c>
+      <c r="B106" s="7"/>
+      <c r="C106" s="7"/>
+      <c r="D106" s="256">
+        <v>28000</v>
+      </c>
+      <c r="E106" s="149">
+        <f>D106*91.91%</f>
+        <v>25734.799999999999</v>
+      </c>
+      <c r="F106" s="134">
+        <f>D106*8.09%</f>
+        <v>2265.1999999999998</v>
+      </c>
+      <c r="H106" s="150"/>
+      <c r="J106" s="113"/>
+    </row>
+    <row r="107" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A107" s="7"/>
+      <c r="B107" s="7"/>
+      <c r="C107" s="7"/>
+      <c r="D107" s="185"/>
+      <c r="E107" s="116"/>
+      <c r="F107" s="7"/>
+      <c r="H107" s="150"/>
+      <c r="J107" s="109"/>
+    </row>
+    <row r="108" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A108" s="95" t="s">
+        <v>101</v>
+      </c>
+      <c r="B108" s="95"/>
+      <c r="C108" s="95"/>
+      <c r="D108" s="107">
+        <f>SUM(D105:D107)</f>
+        <v>250264.92</v>
+      </c>
+      <c r="E108" s="107">
+        <f>SUM(E105:E107)</f>
+        <v>230018.48797199997</v>
+      </c>
+      <c r="F108" s="107">
+        <f>SUM(F105:F107)</f>
+        <v>20246.432028000003</v>
+      </c>
+      <c r="G108" s="109">
+        <f>E108+F108</f>
+        <v>250264.91999999998</v>
+      </c>
+      <c r="H108" s="150" t="str">
+        <f>IF(D108=G108, "", "Error")</f>
+        <v/>
+      </c>
+      <c r="J108" s="109"/>
+    </row>
+    <row r="109" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A109" s="7"/>
+      <c r="B109" s="7"/>
+      <c r="C109" s="7"/>
+      <c r="D109" s="113"/>
+      <c r="E109" s="117"/>
+      <c r="F109" s="7"/>
+      <c r="H109" s="150"/>
+    </row>
+    <row r="110" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A110" s="94" t="s">
+        <v>102</v>
+      </c>
+      <c r="B110" s="7"/>
+      <c r="C110" s="7"/>
+      <c r="D110" s="113">
+        <v>100104.56</v>
+      </c>
+      <c r="E110" s="149">
+        <f>D110*91.91%</f>
+        <v>92006.101095999984</v>
+      </c>
+      <c r="F110" s="134">
+        <f>D110*8.09%</f>
+        <v>8098.4589040000001</v>
+      </c>
+      <c r="H110" s="150"/>
+    </row>
+    <row r="111" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A111" s="94" t="s">
         <v>103</v>
       </c>
-      <c r="B104" s="7"/>
-      <c r="C104" s="122"/>
-      <c r="D104" s="113">
+      <c r="B111" s="7"/>
+      <c r="C111" s="122"/>
+      <c r="D111" s="113">
         <v>44400</v>
       </c>
-      <c r="E104" s="149">
-        <f>D104*91.91%</f>
+      <c r="E111" s="149">
+        <f>D111*91.91%</f>
         <v>40808.039999999994</v>
       </c>
-      <c r="F104" s="134">
-        <f>D104*8.09%</f>
+      <c r="F111" s="134">
+        <f>D111*8.09%</f>
         <v>3591.96</v>
       </c>
-      <c r="H104" s="150"/>
-    </row>
-    <row r="105" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A105" s="95" t="s">
+      <c r="H111" s="150"/>
+    </row>
+    <row r="112" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A112" s="95" t="s">
         <v>15</v>
       </c>
-      <c r="B105" s="95"/>
-      <c r="C105" s="95"/>
-      <c r="D105" s="158">
-        <f>SUM(D103:D104)</f>
+      <c r="B112" s="95"/>
+      <c r="C112" s="95"/>
+      <c r="D112" s="158">
+        <f>SUM(D110:D111)</f>
         <v>144504.56</v>
       </c>
-      <c r="E105" s="147">
-        <f t="shared" ref="E105:F105" si="26">SUM(E103:E104)</f>
+      <c r="E112" s="147">
+        <f t="shared" ref="E112:F112" si="26">SUM(E110:E111)</f>
         <v>132814.14109599998</v>
       </c>
-      <c r="F105" s="147">
+      <c r="F112" s="147">
         <f t="shared" si="26"/>
         <v>11690.418904</v>
       </c>
-      <c r="G105" s="109">
-        <f>E105+F105</f>
+      <c r="G112" s="109">
+        <f>E112+F112</f>
         <v>144504.55999999997</v>
       </c>
-      <c r="H105" s="150" t="str">
-        <f>IF(D105=G105, "", "Error")</f>
+      <c r="H112" s="150" t="str">
+        <f>IF(D112=G112, "", "Error")</f>
         <v/>
       </c>
     </row>
-    <row r="106" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A106" s="7"/>
-      <c r="B106" s="7"/>
-      <c r="C106" s="7"/>
-      <c r="D106" s="186"/>
-      <c r="E106" s="12"/>
-      <c r="F106" s="7"/>
-      <c r="H106" s="150"/>
-    </row>
-    <row r="107" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A107" s="99" t="s">
+    <row r="113" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A113" s="7"/>
+      <c r="B113" s="7"/>
+      <c r="C113" s="7"/>
+      <c r="D113" s="186"/>
+      <c r="E113" s="12"/>
+      <c r="F113" s="7"/>
+      <c r="H113" s="150"/>
+    </row>
+    <row r="114" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A114" s="99" t="s">
         <v>134</v>
       </c>
-      <c r="B107" s="99"/>
-      <c r="C107" s="99"/>
-      <c r="D107" s="187"/>
-      <c r="E107" s="118">
-        <f>D107*91.91%</f>
-        <v>0</v>
-      </c>
-      <c r="F107" s="136">
-        <f>D107*8.09%</f>
-        <v>0</v>
-      </c>
-      <c r="G107" s="109">
-        <f>E107+F107</f>
-        <v>0</v>
-      </c>
-      <c r="H107" s="150" t="str">
-        <f>IF(D107=G107, "", "Error")</f>
+      <c r="B114" s="99"/>
+      <c r="C114" s="99"/>
+      <c r="D114" s="187"/>
+      <c r="E114" s="118">
+        <f>D114*91.91%</f>
+        <v>0</v>
+      </c>
+      <c r="F114" s="136">
+        <f>D114*8.09%</f>
+        <v>0</v>
+      </c>
+      <c r="G114" s="109">
+        <f>E114+F114</f>
+        <v>0</v>
+      </c>
+      <c r="H114" s="150" t="str">
+        <f>IF(D114=G114, "", "Error")</f>
         <v/>
       </c>
     </row>
-    <row r="108" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A108" s="1"/>
-      <c r="D108" s="184"/>
-      <c r="E108" s="2"/>
-      <c r="F108" s="10"/>
-      <c r="G108" s="157"/>
-      <c r="H108" s="150"/>
-    </row>
-    <row r="109" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A109" s="4" t="s">
+    <row r="115" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A115" s="1"/>
+      <c r="D115" s="184"/>
+      <c r="E115" s="2"/>
+      <c r="F115" s="10"/>
+      <c r="G115" s="157"/>
+      <c r="H115" s="150"/>
+    </row>
+    <row r="116" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A116" s="4" t="s">
         <v>104</v>
       </c>
-      <c r="B109" s="60"/>
-      <c r="C109" s="5"/>
-      <c r="D109" s="188">
-        <f>SUM(D107+D105+D101+D94+D88+D55+D35+D30+D48)</f>
-        <v>7496328.3699999992</v>
-      </c>
-      <c r="E109" s="148">
-        <f>SUM(E107+E105+E101+E94+E88+E55+E35+E30+E48)</f>
-        <v>7082805.3203670001</v>
-      </c>
-      <c r="F109" s="148">
-        <f>SUM(F107+F105+F101+F94+F88+F55+F35+F30+F48)</f>
-        <v>413523.04963299993</v>
-      </c>
-      <c r="G109" s="109">
-        <f>E109+F109</f>
-        <v>7496328.3700000001</v>
-      </c>
-      <c r="H109" s="150" t="str">
-        <f>IF(D109=G109, "", "Error")</f>
-        <v/>
-      </c>
-      <c r="I109" s="178">
-        <f>D109-G109</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="110" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="D110" s="184"/>
-      <c r="E110" s="109"/>
-    </row>
-    <row r="111" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A111" s="142" t="s">
+      <c r="B116" s="60"/>
+      <c r="C116" s="5"/>
+      <c r="D116" s="188">
+        <f>SUM(D114+D112+D108+D101+D95+D55+D35+D30+D48)</f>
+        <v>10659184.91</v>
+      </c>
+      <c r="E116" s="148">
+        <f>SUM(E114+E112+E108+E101+E95+E55+E35+E30+E48)</f>
+        <v>10095751.311878001</v>
+      </c>
+      <c r="F116" s="148">
+        <f>SUM(F114+F112+F108+F101+F95+F55+F35+F30+F48)</f>
+        <v>577995.59812199988</v>
+      </c>
+      <c r="G116" s="109">
+        <f>E116+F116</f>
+        <v>10673746.910000002</v>
+      </c>
+      <c r="H116" s="150" t="str">
+        <f>IF(D116=G116, "", "Error")</f>
+        <v>Error</v>
+      </c>
+      <c r="I116" s="178">
+        <f>D116-G116</f>
+        <v>-14562.000000001863</v>
+      </c>
+    </row>
+    <row r="117" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D117" s="184"/>
+      <c r="E117" s="109"/>
+    </row>
+    <row r="118" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A118" s="142" t="s">
         <v>121</v>
       </c>
-      <c r="B111" s="141"/>
-      <c r="C111" s="141"/>
-      <c r="E111" s="109"/>
-    </row>
-    <row r="112" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A112" s="1"/>
-      <c r="C112" s="139"/>
-      <c r="E112" s="109"/>
-    </row>
-    <row r="113" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A113" s="1"/>
-      <c r="C113" s="139"/>
-      <c r="E113" s="109"/>
-    </row>
-    <row r="114" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A114" s="143" t="s">
+      <c r="B118" s="141"/>
+      <c r="C118" s="141"/>
+      <c r="E118" s="109"/>
+    </row>
+    <row r="119" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A119" s="1"/>
+      <c r="C119" s="139"/>
+      <c r="E119" s="109"/>
+    </row>
+    <row r="120" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A120" s="1"/>
+      <c r="C120" s="139"/>
+      <c r="E120" s="109"/>
+    </row>
+    <row r="121" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A121" s="143" t="s">
         <v>30</v>
       </c>
-      <c r="B114" s="144"/>
-      <c r="C114" s="140">
-        <f>SUM(C112:C113)</f>
-        <v>0</v>
-      </c>
-      <c r="E114" s="109"/>
-    </row>
-    <row r="115" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="E115" s="109"/>
-    </row>
-    <row r="116" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="E116" s="137"/>
-    </row>
-    <row r="117" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A117" s="223" t="s">
+      <c r="B121" s="144"/>
+      <c r="C121" s="140">
+        <f>SUM(C119:C120)</f>
+        <v>0</v>
+      </c>
+      <c r="E121" s="109"/>
+    </row>
+    <row r="122" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="E122" s="109"/>
+    </row>
+    <row r="123" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="E123" s="137"/>
+    </row>
+    <row r="124" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A124" s="228" t="s">
         <v>114</v>
       </c>
-      <c r="B117" s="224"/>
-      <c r="C117" s="224"/>
-      <c r="D117" s="224"/>
-      <c r="E117" s="171" t="s">
+      <c r="B124" s="229"/>
+      <c r="C124" s="229"/>
+      <c r="D124" s="229"/>
+      <c r="E124" s="171" t="s">
         <v>22</v>
       </c>
-      <c r="F117" s="172" t="s">
+      <c r="F124" s="172" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="118" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A118" s="220"/>
-      <c r="B118" s="221"/>
-      <c r="C118" s="222"/>
-      <c r="D118" s="166"/>
-      <c r="E118" s="149"/>
-      <c r="F118" s="134"/>
-    </row>
-    <row r="119" spans="1:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A119" s="217" t="s">
-        <v>160</v>
-      </c>
-      <c r="B119" s="218"/>
-      <c r="C119" s="173"/>
-      <c r="D119" s="113">
+    <row r="125" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A125" s="225"/>
+      <c r="B125" s="226"/>
+      <c r="C125" s="227"/>
+      <c r="D125" s="166"/>
+      <c r="E125" s="149"/>
+      <c r="F125" s="134"/>
+    </row>
+    <row r="126" spans="1:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A126" s="222" t="s">
+        <v>152</v>
+      </c>
+      <c r="B126" s="223"/>
+      <c r="C126" s="173"/>
+      <c r="D126" s="113">
         <v>300000</v>
       </c>
-      <c r="E119" s="149">
-        <f t="shared" ref="E119:E120" si="27">D119*91.91%</f>
+      <c r="E126" s="149">
+        <f t="shared" ref="E126:E127" si="27">D126*91.91%</f>
         <v>275730</v>
       </c>
-      <c r="F119" s="134">
-        <f t="shared" ref="F119:F120" si="28">D119*8.09%</f>
+      <c r="F126" s="134">
+        <f t="shared" ref="F126:F127" si="28">D126*8.09%</f>
         <v>24270</v>
       </c>
     </row>
-    <row r="120" spans="1:9" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A120" s="217" t="s">
-        <v>153</v>
-      </c>
-      <c r="B120" s="218"/>
-      <c r="C120" s="173"/>
-      <c r="D120" s="113">
+    <row r="127" spans="1:9" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A127" s="222" t="s">
+        <v>146</v>
+      </c>
+      <c r="B127" s="223"/>
+      <c r="C127" s="173"/>
+      <c r="D127" s="113">
         <v>10391.24</v>
       </c>
-      <c r="E120" s="149">
+      <c r="E127" s="149">
         <f t="shared" si="27"/>
         <v>9550.5886839999985</v>
       </c>
-      <c r="F120" s="134">
+      <c r="F127" s="134">
         <f t="shared" si="28"/>
         <v>840.65131599999995</v>
       </c>
     </row>
-    <row r="121" spans="1:9" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A121" s="217"/>
-      <c r="B121" s="218"/>
-      <c r="C121" s="219"/>
-      <c r="D121" s="113"/>
-      <c r="E121" s="149">
-        <f>D121*91.91%</f>
-        <v>0</v>
-      </c>
-      <c r="F121" s="134">
-        <f>D121*8.09%</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="122" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A122" s="211" t="s">
+    <row r="128" spans="1:9" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A128" s="222"/>
+      <c r="B128" s="223"/>
+      <c r="C128" s="224"/>
+      <c r="D128" s="113"/>
+      <c r="E128" s="149">
+        <f>D128*91.91%</f>
+        <v>0</v>
+      </c>
+      <c r="F128" s="134">
+        <f>D128*8.09%</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="129" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A129" s="216" t="s">
         <v>30</v>
       </c>
-      <c r="B122" s="212"/>
-      <c r="C122" s="213"/>
-      <c r="D122" s="170">
-        <f>SUM(D118:D121)</f>
+      <c r="B129" s="217"/>
+      <c r="C129" s="218"/>
+      <c r="D129" s="170">
+        <f>SUM(D125:D128)</f>
         <v>310391.24</v>
       </c>
-      <c r="E122" s="170">
-        <f>SUM(E118:E121)</f>
+      <c r="E129" s="170">
+        <f>SUM(E125:E128)</f>
         <v>285280.58868400002</v>
       </c>
-      <c r="F122" s="170">
-        <f>SUM(F118:F121)</f>
+      <c r="F129" s="170">
+        <f>SUM(F125:F128)</f>
         <v>25110.651315999999</v>
       </c>
-      <c r="H122" s="109">
-        <f>E122+F122</f>
+      <c r="H129" s="109">
+        <f>E129+F129</f>
         <v>310391.24</v>
       </c>
-      <c r="I122" s="150" t="str">
-        <f>IF(D122=H122, "", "Error")</f>
+      <c r="I129" s="150" t="str">
+        <f>IF(D129=H129, "", "Error")</f>
         <v/>
       </c>
     </row>
-    <row r="124" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="E124" s="109"/>
-    </row>
-    <row r="125" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A125" s="102" t="s">
+    <row r="131" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="E131" s="109"/>
+    </row>
+    <row r="132" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A132" s="102" t="s">
         <v>105</v>
       </c>
-      <c r="B125" s="103">
-        <f>D109</f>
-        <v>7496328.3699999992</v>
-      </c>
-    </row>
-    <row r="126" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A126" s="104" t="s">
+      <c r="B132" s="103">
+        <f>D116</f>
+        <v>10659184.91</v>
+      </c>
+    </row>
+    <row r="133" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A133" s="104" t="s">
         <v>107</v>
       </c>
-      <c r="B126" s="105">
-        <f>D109-D107</f>
-        <v>7496328.3699999992</v>
-      </c>
-    </row>
-    <row r="127" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="D127" s="235"/>
-      <c r="E127" s="235"/>
-    </row>
-    <row r="128" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A128" s="74" t="s">
+      <c r="B133" s="105">
+        <f>D116-D114</f>
+        <v>10659184.91</v>
+      </c>
+    </row>
+    <row r="134" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="D134" s="206"/>
+      <c r="E134" s="206"/>
+    </row>
+    <row r="135" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A135" s="74" t="s">
         <v>91</v>
       </c>
-      <c r="B128" s="75"/>
-      <c r="C128" s="76"/>
-      <c r="D128" s="235"/>
-      <c r="E128" s="235"/>
-    </row>
-    <row r="129" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A129" s="77" t="s">
+      <c r="B135" s="75"/>
+      <c r="C135" s="76"/>
+      <c r="D135" s="206"/>
+      <c r="E135" s="206"/>
+    </row>
+    <row r="136" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A136" s="77" t="s">
         <v>92</v>
       </c>
-      <c r="B129" s="78">
+      <c r="B136" s="78">
         <v>6056324.5665496523</v>
       </c>
-      <c r="C129" s="78"/>
-      <c r="D129" s="235"/>
-      <c r="E129" s="235"/>
-    </row>
-    <row r="130" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A130" s="79" t="s">
+      <c r="C136" s="78"/>
+      <c r="D136" s="206"/>
+      <c r="E136" s="206"/>
+    </row>
+    <row r="137" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A137" s="79" t="s">
         <v>93</v>
       </c>
-      <c r="B130" s="92">
+      <c r="B137" s="92">
         <f>PRORRATEO!G52</f>
         <v>6320855.3670509998</v>
       </c>
-      <c r="C130" s="78" t="s">
+      <c r="C137" s="78" t="s">
         <v>94</v>
       </c>
-      <c r="D130" s="235"/>
-      <c r="E130" s="235"/>
-    </row>
-    <row r="131" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A131" s="79" t="s">
+      <c r="D137" s="206"/>
+      <c r="E137" s="206"/>
+    </row>
+    <row r="138" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A138" s="79" t="s">
         <v>116</v>
       </c>
-      <c r="B131" s="175">
-        <f>-B126</f>
-        <v>-7496328.3699999992</v>
-      </c>
-      <c r="C131" s="76"/>
-      <c r="D131" s="235"/>
-      <c r="E131" s="235"/>
-      <c r="G131" s="113"/>
-    </row>
-    <row r="132" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A132" s="79" t="s">
+      <c r="B138" s="175">
+        <f>-B133</f>
+        <v>-10659184.91</v>
+      </c>
+      <c r="C138" s="76"/>
+      <c r="D138" s="206"/>
+      <c r="E138" s="206"/>
+      <c r="G138" s="113"/>
+    </row>
+    <row r="139" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A139" s="79" t="s">
         <v>115</v>
       </c>
-      <c r="B132" s="175">
-        <f>-D122</f>
+      <c r="B139" s="175">
+        <f>-D129</f>
         <v>-310391.24</v>
       </c>
-      <c r="C132" s="76"/>
-      <c r="D132" s="235"/>
-      <c r="E132" s="235"/>
-      <c r="G132" s="125"/>
-    </row>
-    <row r="133" spans="1:7" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A133" s="201" t="s">
-        <v>168</v>
-      </c>
-      <c r="B133" s="175">
+      <c r="C139" s="76"/>
+      <c r="D139" s="206"/>
+      <c r="E139" s="206"/>
+      <c r="G139" s="125"/>
+    </row>
+    <row r="140" spans="1:9" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A140" s="201" t="s">
+        <v>158</v>
+      </c>
+      <c r="B140" s="175">
         <v>-338000</v>
       </c>
-      <c r="C133" s="76"/>
-      <c r="D133" s="198"/>
-      <c r="E133" s="198"/>
-      <c r="G133" s="125"/>
-    </row>
-    <row r="134" spans="1:7" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A134" s="200" t="s">
-        <v>175</v>
-      </c>
-      <c r="B134" s="175">
+      <c r="C140" s="76"/>
+      <c r="D140" s="198"/>
+      <c r="E140" s="198"/>
+      <c r="G140" s="125"/>
+    </row>
+    <row r="141" spans="1:9" ht="48" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A141" s="200" t="s">
+        <v>165</v>
+      </c>
+      <c r="B141" s="175">
         <v>-308000</v>
       </c>
-      <c r="C134" s="76"/>
-      <c r="D134" s="198"/>
-      <c r="E134" s="198"/>
-      <c r="G134" s="125"/>
-    </row>
-    <row r="135" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A135" s="79" t="s">
+      <c r="C141" s="76"/>
+      <c r="D141" s="198"/>
+      <c r="E141" s="198"/>
+      <c r="G141" s="125"/>
+    </row>
+    <row r="142" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A142" s="79" t="s">
         <v>106</v>
       </c>
-      <c r="B135" s="175">
-        <f>-B142</f>
-        <v>0</v>
-      </c>
-      <c r="C135" s="80"/>
-    </row>
-    <row r="136" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A136" s="79" t="s">
+      <c r="B142" s="175">
+        <f>-B149</f>
+        <v>0</v>
+      </c>
+      <c r="C142" s="80"/>
+    </row>
+    <row r="143" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A143" s="79" t="s">
         <v>121</v>
       </c>
-      <c r="B136" s="93">
-        <f>-C114</f>
-        <v>0</v>
-      </c>
-      <c r="C136" s="80"/>
-    </row>
-    <row r="137" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A137" s="79"/>
-      <c r="B137" s="75"/>
-      <c r="C137" s="80"/>
-    </row>
-    <row r="138" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A138" s="77" t="s">
+      <c r="B143" s="93">
+        <f>-C121</f>
+        <v>0</v>
+      </c>
+      <c r="C143" s="80"/>
+    </row>
+    <row r="144" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A144" s="79"/>
+      <c r="B144" s="75"/>
+      <c r="C144" s="80"/>
+    </row>
+    <row r="145" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A145" s="77" t="s">
         <v>95</v>
       </c>
-      <c r="B138" s="81">
-        <f>SUM(B129:B137)</f>
-        <v>3924460.3236006536</v>
-      </c>
-      <c r="C138" s="154"/>
-    </row>
-    <row r="139" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A139" s="80"/>
-      <c r="C139" s="76"/>
-      <c r="D139" s="83"/>
-    </row>
-    <row r="140" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C140" s="76"/>
-      <c r="D140" s="109"/>
-      <c r="E140" s="178"/>
-    </row>
-    <row r="141" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A141" s="74" t="s">
+      <c r="B145" s="81">
+        <f>SUM(B136:B144)</f>
+        <v>761603.78360065282</v>
+      </c>
+      <c r="C145" s="154"/>
+    </row>
+    <row r="146" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A146" s="80"/>
+      <c r="C146" s="76"/>
+      <c r="D146" s="83"/>
+    </row>
+    <row r="147" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="C147" s="76"/>
+      <c r="D147" s="109"/>
+      <c r="E147" s="178"/>
+    </row>
+    <row r="148" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A148" s="74" t="s">
         <v>96</v>
       </c>
-      <c r="B141" s="11">
+      <c r="B148" s="11">
         <v>-310694.54000000004</v>
       </c>
-      <c r="C141" s="82"/>
-      <c r="D141" s="178"/>
-      <c r="E141" s="178"/>
-      <c r="F141" s="178"/>
-    </row>
-    <row r="142" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A142" s="77" t="s">
-        <v>176</v>
-      </c>
-      <c r="B142" s="93"/>
-      <c r="C142" s="82"/>
-      <c r="D142" s="178"/>
-      <c r="E142" s="199"/>
-    </row>
-    <row r="143" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A143" s="77"/>
-      <c r="B143" s="175"/>
-      <c r="C143" s="82"/>
-      <c r="E143" s="109"/>
-    </row>
-    <row r="144" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A144" s="77" t="s">
-        <v>163</v>
-      </c>
-      <c r="B144" s="175">
+      <c r="C148" s="82"/>
+      <c r="D148" s="178"/>
+      <c r="E148" s="178"/>
+      <c r="F148" s="178"/>
+    </row>
+    <row r="149" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A149" s="77" t="s">
+        <v>166</v>
+      </c>
+      <c r="B149" s="93"/>
+      <c r="C149" s="82"/>
+      <c r="D149" s="178"/>
+      <c r="E149" s="199"/>
+    </row>
+    <row r="150" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A150" s="77"/>
+      <c r="B150" s="175"/>
+      <c r="C150" s="82"/>
+      <c r="E150" s="109"/>
+    </row>
+    <row r="151" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A151" s="77" t="s">
+        <v>155</v>
+      </c>
+      <c r="B151" s="175">
         <v>-55000</v>
       </c>
-      <c r="C144" s="82"/>
-      <c r="E144" s="109"/>
-    </row>
-    <row r="145" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A145" s="100" t="s">
+      <c r="C151" s="82"/>
+      <c r="E151" s="109"/>
+    </row>
+    <row r="152" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A152" s="100" t="s">
         <v>30</v>
       </c>
-      <c r="B145" s="101">
-        <f>SUM(B141:B144)</f>
+      <c r="B152" s="101">
+        <f>SUM(B148:B151)</f>
         <v>-365694.54000000004</v>
       </c>
-      <c r="C145" s="82"/>
-    </row>
-    <row r="146" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="C146" s="83"/>
-      <c r="D146" s="178"/>
-    </row>
-    <row r="147" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="B147" s="80"/>
-      <c r="C147" s="76"/>
-    </row>
-    <row r="149" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="N149" s="12"/>
-    </row>
-    <row r="152" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="B152" s="234" t="s">
-        <v>174</v>
-      </c>
-      <c r="C152" s="234"/>
-      <c r="D152" s="234"/>
-      <c r="E152" s="234"/>
+      <c r="C152" s="82"/>
     </row>
     <row r="153" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="B153" s="234"/>
-      <c r="C153" s="234"/>
-      <c r="D153" s="234"/>
-      <c r="E153" s="234"/>
+      <c r="C153" s="83"/>
+      <c r="D153" s="178"/>
     </row>
     <row r="154" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="B154" s="234"/>
-      <c r="C154" s="234"/>
-      <c r="D154" s="234"/>
-      <c r="E154" s="234"/>
-    </row>
-    <row r="155" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="B155" s="234"/>
-      <c r="C155" s="234"/>
-      <c r="D155" s="234"/>
-      <c r="E155" s="234"/>
+      <c r="B154" s="80"/>
+      <c r="C154" s="76"/>
     </row>
     <row r="156" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="B156" s="234"/>
-      <c r="C156" s="234"/>
-      <c r="D156" s="234"/>
-      <c r="E156" s="234"/>
+      <c r="N156" s="12"/>
+    </row>
+    <row r="159" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="B159" s="205" t="s">
+        <v>164</v>
+      </c>
+      <c r="C159" s="205"/>
+      <c r="D159" s="205"/>
+      <c r="E159" s="205"/>
+    </row>
+    <row r="160" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="B160" s="205"/>
+      <c r="C160" s="205"/>
+      <c r="D160" s="205"/>
+      <c r="E160" s="205"/>
+    </row>
+    <row r="161" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B161" s="205"/>
+      <c r="C161" s="205"/>
+      <c r="D161" s="205"/>
+      <c r="E161" s="205"/>
+    </row>
+    <row r="162" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B162" s="205"/>
+      <c r="C162" s="205"/>
+      <c r="D162" s="205"/>
+      <c r="E162" s="205"/>
+    </row>
+    <row r="163" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B163" s="205"/>
+      <c r="C163" s="205"/>
+      <c r="D163" s="205"/>
+      <c r="E163" s="205"/>
     </row>
   </sheetData>
-  <mergeCells count="19">
-    <mergeCell ref="A71:C71"/>
-    <mergeCell ref="B152:E156"/>
-    <mergeCell ref="D127:E132"/>
+  <mergeCells count="20">
+    <mergeCell ref="A76:C76"/>
+    <mergeCell ref="A127:B127"/>
+    <mergeCell ref="A126:B126"/>
+    <mergeCell ref="A88:C88"/>
+    <mergeCell ref="A72:C72"/>
+    <mergeCell ref="B159:E163"/>
+    <mergeCell ref="D134:E139"/>
     <mergeCell ref="B14:D17"/>
-    <mergeCell ref="A122:C122"/>
+    <mergeCell ref="A129:C129"/>
+    <mergeCell ref="A67:C67"/>
+    <mergeCell ref="A128:C128"/>
+    <mergeCell ref="A125:C125"/>
+    <mergeCell ref="A124:D124"/>
+    <mergeCell ref="A75:C75"/>
     <mergeCell ref="A66:C66"/>
-    <mergeCell ref="A121:C121"/>
-    <mergeCell ref="A118:C118"/>
-    <mergeCell ref="A117:D117"/>
-    <mergeCell ref="A74:C74"/>
-    <mergeCell ref="A65:C65"/>
-    <mergeCell ref="A72:C72"/>
-    <mergeCell ref="A67:C67"/>
+    <mergeCell ref="A73:C73"/>
     <mergeCell ref="A68:C68"/>
     <mergeCell ref="A69:C69"/>
     <mergeCell ref="A70:C70"/>
-    <mergeCell ref="A75:C75"/>
-    <mergeCell ref="A120:B120"/>
-    <mergeCell ref="A119:B119"/>
+    <mergeCell ref="A71:C71"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="landscape" r:id="rId1"/>
@@ -4632,15 +4861,15 @@
       <c r="K1" s="8" t="s">
         <v>125</v>
       </c>
-      <c r="L1" s="243">
-        <f>RESUMEN!D109</f>
-        <v>7496328.3699999992</v>
-      </c>
-      <c r="M1" s="244"/>
+      <c r="L1" s="239">
+        <f>RESUMEN!D116</f>
+        <v>10659184.91</v>
+      </c>
+      <c r="M1" s="240"/>
       <c r="N1" s="152"/>
       <c r="O1" s="135">
         <f>L1*8.09%</f>
-        <v>606452.96513299993</v>
+        <v>862328.05921900005</v>
       </c>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.25">
@@ -4665,7 +4894,7 @@
       <c r="N2" s="153"/>
       <c r="O2" s="135">
         <f>O1-K7-553-50-86-8</f>
-        <v>207324.22721099993</v>
+        <v>463199.32129700005</v>
       </c>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.25">
@@ -4687,7 +4916,7 @@
       </c>
       <c r="L3" s="8"/>
       <c r="M3" s="128">
-        <f>RESUMEN!D122</f>
+        <f>RESUMEN!D129</f>
         <v>310391.24</v>
       </c>
       <c r="N3" s="151"/>
@@ -4721,13 +4950,13 @@
       <c r="A5" s="236" t="s">
         <v>20</v>
       </c>
-      <c r="B5" s="238" t="s">
+      <c r="B5" s="250" t="s">
         <v>21</v>
       </c>
       <c r="C5" s="236" t="s">
         <v>22</v>
       </c>
-      <c r="D5" s="240" t="s">
+      <c r="D5" s="248" t="s">
         <v>23</v>
       </c>
       <c r="E5" s="236" t="s">
@@ -4739,43 +4968,43 @@
       <c r="G5" s="236" t="s">
         <v>25</v>
       </c>
-      <c r="H5" s="247" t="s">
+      <c r="H5" s="243" t="s">
         <v>26</v>
       </c>
-      <c r="I5" s="240" t="s">
+      <c r="I5" s="248" t="s">
         <v>109</v>
       </c>
-      <c r="J5" s="245" t="s">
+      <c r="J5" s="241" t="s">
         <v>27</v>
       </c>
-      <c r="K5" s="245" t="s">
+      <c r="K5" s="241" t="s">
         <v>70</v>
       </c>
-      <c r="L5" s="250" t="s">
+      <c r="L5" s="246" t="s">
         <v>124</v>
       </c>
-      <c r="M5" s="245" t="s">
+      <c r="M5" s="241" t="s">
         <v>68</v>
       </c>
-      <c r="N5" s="245" t="s">
+      <c r="N5" s="241" t="s">
         <v>69</v>
       </c>
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A6" s="237"/>
-      <c r="B6" s="239"/>
+      <c r="B6" s="251"/>
       <c r="C6" s="237"/>
-      <c r="D6" s="241"/>
+      <c r="D6" s="252"/>
       <c r="E6" s="237"/>
       <c r="F6" s="237"/>
       <c r="G6" s="237"/>
-      <c r="H6" s="248"/>
-      <c r="I6" s="252"/>
-      <c r="J6" s="246"/>
-      <c r="K6" s="249"/>
-      <c r="L6" s="251"/>
-      <c r="M6" s="249"/>
-      <c r="N6" s="246"/>
+      <c r="H6" s="244"/>
+      <c r="I6" s="249"/>
+      <c r="J6" s="242"/>
+      <c r="K6" s="245"/>
+      <c r="L6" s="247"/>
+      <c r="M6" s="245"/>
+      <c r="N6" s="242"/>
     </row>
     <row r="7" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A7" s="7" t="s">
@@ -4889,7 +5118,7 @@
         <v>222096.62408426331</v>
       </c>
       <c r="G9" s="192">
-        <f>250969-G34+RESUMEN!D65</f>
+        <f>250969-G34+RESUMEN!D66</f>
         <v>333122.69579999999</v>
       </c>
       <c r="H9" s="131">
@@ -5574,7 +5803,7 @@
         <v>385103.52163409517</v>
       </c>
       <c r="G23" s="192">
-        <f>447000-G46+RESUMEN!D70+RESUMEN!D71</f>
+        <f>447000-G46+RESUMEN!D71+RESUMEN!D72</f>
         <v>582942.08675000002</v>
       </c>
       <c r="H23" s="131">
@@ -5818,7 +6047,7 @@
         <v>314286.41577654087</v>
       </c>
       <c r="G28" s="191">
-        <f>371000-G32-G33+RESUMEN!D73</f>
+        <f>371000-G32-G33+RESUMEN!D74</f>
         <v>413583.78619999997</v>
       </c>
       <c r="H28" s="131">
@@ -5867,7 +6096,7 @@
         <v>325490.37115669996</v>
       </c>
       <c r="G29" s="192">
-        <f>401000-G42-G43-G44+RESUMEN!D72</f>
+        <f>401000-G42-G43-G44+RESUMEN!D73</f>
         <v>413311.71970000002</v>
       </c>
       <c r="H29" s="132">
@@ -6557,7 +6786,7 @@
       </c>
       <c r="P43" s="109">
         <f>L1-K52</f>
-        <v>1105640.362077998</v>
+        <v>4268496.902077999</v>
       </c>
     </row>
     <row r="44" spans="1:17" x14ac:dyDescent="0.25">
@@ -6989,36 +7218,36 @@
     <row r="53" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="K53" s="138">
         <f>K52-L1</f>
-        <v>-1105640.362077998</v>
+        <v>-4268496.902077999</v>
       </c>
     </row>
     <row r="54" spans="1:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C54" s="242"/>
-      <c r="D54" s="242"/>
-      <c r="E54" s="242"/>
-      <c r="F54" s="242"/>
-      <c r="G54" s="242"/>
-      <c r="H54" s="242"/>
-      <c r="I54" s="242"/>
-      <c r="J54" s="242"/>
-      <c r="K54" s="242"/>
-      <c r="L54" s="242"/>
-      <c r="M54" s="242"/>
-      <c r="N54" s="242"/>
+      <c r="C54" s="238"/>
+      <c r="D54" s="238"/>
+      <c r="E54" s="238"/>
+      <c r="F54" s="238"/>
+      <c r="G54" s="238"/>
+      <c r="H54" s="238"/>
+      <c r="I54" s="238"/>
+      <c r="J54" s="238"/>
+      <c r="K54" s="238"/>
+      <c r="L54" s="238"/>
+      <c r="M54" s="238"/>
+      <c r="N54" s="238"/>
     </row>
     <row r="55" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
-      <c r="C55" s="242"/>
-      <c r="D55" s="242"/>
-      <c r="E55" s="242"/>
-      <c r="F55" s="242"/>
-      <c r="G55" s="242"/>
-      <c r="H55" s="242"/>
-      <c r="I55" s="242"/>
-      <c r="J55" s="242"/>
-      <c r="K55" s="242"/>
-      <c r="L55" s="242"/>
-      <c r="M55" s="242"/>
-      <c r="N55" s="242"/>
+      <c r="C55" s="238"/>
+      <c r="D55" s="238"/>
+      <c r="E55" s="238"/>
+      <c r="F55" s="238"/>
+      <c r="G55" s="238"/>
+      <c r="H55" s="238"/>
+      <c r="I55" s="238"/>
+      <c r="J55" s="238"/>
+      <c r="K55" s="238"/>
+      <c r="L55" s="238"/>
+      <c r="M55" s="238"/>
+      <c r="N55" s="238"/>
     </row>
     <row r="56" spans="1:16" x14ac:dyDescent="0.25">
       <c r="C56" s="168"/>
@@ -7035,107 +7264,112 @@
       <c r="N56" s="168"/>
     </row>
     <row r="57" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="C57" s="242" t="s">
+      <c r="C57" s="238" t="s">
         <v>130</v>
       </c>
-      <c r="D57" s="242"/>
-      <c r="E57" s="242"/>
-      <c r="F57" s="242"/>
-      <c r="G57" s="242"/>
-      <c r="H57" s="242"/>
-      <c r="I57" s="242"/>
-      <c r="J57" s="242"/>
-      <c r="K57" s="242"/>
-      <c r="L57" s="242"/>
-      <c r="M57" s="242"/>
-      <c r="N57" s="242"/>
+      <c r="D57" s="238"/>
+      <c r="E57" s="238"/>
+      <c r="F57" s="238"/>
+      <c r="G57" s="238"/>
+      <c r="H57" s="238"/>
+      <c r="I57" s="238"/>
+      <c r="J57" s="238"/>
+      <c r="K57" s="238"/>
+      <c r="L57" s="238"/>
+      <c r="M57" s="238"/>
+      <c r="N57" s="238"/>
     </row>
     <row r="58" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="C58" s="242"/>
-      <c r="D58" s="242"/>
-      <c r="E58" s="242"/>
-      <c r="F58" s="242"/>
-      <c r="G58" s="242"/>
-      <c r="H58" s="242"/>
-      <c r="I58" s="242"/>
-      <c r="J58" s="242"/>
-      <c r="K58" s="242"/>
-      <c r="L58" s="242"/>
-      <c r="M58" s="242"/>
-      <c r="N58" s="242"/>
+      <c r="C58" s="238"/>
+      <c r="D58" s="238"/>
+      <c r="E58" s="238"/>
+      <c r="F58" s="238"/>
+      <c r="G58" s="238"/>
+      <c r="H58" s="238"/>
+      <c r="I58" s="238"/>
+      <c r="J58" s="238"/>
+      <c r="K58" s="238"/>
+      <c r="L58" s="238"/>
+      <c r="M58" s="238"/>
+      <c r="N58" s="238"/>
     </row>
     <row r="59" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="C59" s="242"/>
-      <c r="D59" s="242"/>
-      <c r="E59" s="242"/>
-      <c r="F59" s="242"/>
-      <c r="G59" s="242"/>
-      <c r="H59" s="242"/>
-      <c r="I59" s="242"/>
-      <c r="J59" s="242"/>
-      <c r="K59" s="242"/>
-      <c r="L59" s="242"/>
-      <c r="M59" s="242"/>
-      <c r="N59" s="242"/>
+      <c r="C59" s="238"/>
+      <c r="D59" s="238"/>
+      <c r="E59" s="238"/>
+      <c r="F59" s="238"/>
+      <c r="G59" s="238"/>
+      <c r="H59" s="238"/>
+      <c r="I59" s="238"/>
+      <c r="J59" s="238"/>
+      <c r="K59" s="238"/>
+      <c r="L59" s="238"/>
+      <c r="M59" s="238"/>
+      <c r="N59" s="238"/>
     </row>
     <row r="60" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="C60" s="242"/>
-      <c r="D60" s="242"/>
-      <c r="E60" s="242"/>
-      <c r="F60" s="242"/>
-      <c r="G60" s="242"/>
-      <c r="H60" s="242"/>
-      <c r="I60" s="242"/>
-      <c r="J60" s="242"/>
-      <c r="K60" s="242"/>
-      <c r="L60" s="242"/>
-      <c r="M60" s="242"/>
-      <c r="N60" s="242"/>
+      <c r="C60" s="238"/>
+      <c r="D60" s="238"/>
+      <c r="E60" s="238"/>
+      <c r="F60" s="238"/>
+      <c r="G60" s="238"/>
+      <c r="H60" s="238"/>
+      <c r="I60" s="238"/>
+      <c r="J60" s="238"/>
+      <c r="K60" s="238"/>
+      <c r="L60" s="238"/>
+      <c r="M60" s="238"/>
+      <c r="N60" s="238"/>
     </row>
     <row r="61" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="C61" s="242"/>
-      <c r="D61" s="242"/>
-      <c r="E61" s="242"/>
-      <c r="F61" s="242"/>
-      <c r="G61" s="242"/>
-      <c r="H61" s="242"/>
-      <c r="I61" s="242"/>
-      <c r="J61" s="242"/>
-      <c r="K61" s="242"/>
-      <c r="L61" s="242"/>
-      <c r="M61" s="242"/>
-      <c r="N61" s="242"/>
+      <c r="C61" s="238"/>
+      <c r="D61" s="238"/>
+      <c r="E61" s="238"/>
+      <c r="F61" s="238"/>
+      <c r="G61" s="238"/>
+      <c r="H61" s="238"/>
+      <c r="I61" s="238"/>
+      <c r="J61" s="238"/>
+      <c r="K61" s="238"/>
+      <c r="L61" s="238"/>
+      <c r="M61" s="238"/>
+      <c r="N61" s="238"/>
     </row>
     <row r="62" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="C62" s="242"/>
-      <c r="D62" s="242"/>
-      <c r="E62" s="242"/>
-      <c r="F62" s="242"/>
-      <c r="G62" s="242"/>
-      <c r="H62" s="242"/>
-      <c r="I62" s="242"/>
-      <c r="J62" s="242"/>
-      <c r="K62" s="242"/>
-      <c r="L62" s="242"/>
-      <c r="M62" s="242"/>
-      <c r="N62" s="242"/>
+      <c r="C62" s="238"/>
+      <c r="D62" s="238"/>
+      <c r="E62" s="238"/>
+      <c r="F62" s="238"/>
+      <c r="G62" s="238"/>
+      <c r="H62" s="238"/>
+      <c r="I62" s="238"/>
+      <c r="J62" s="238"/>
+      <c r="K62" s="238"/>
+      <c r="L62" s="238"/>
+      <c r="M62" s="238"/>
+      <c r="N62" s="238"/>
     </row>
     <row r="63" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="C63" s="242"/>
-      <c r="D63" s="242"/>
-      <c r="E63" s="242"/>
-      <c r="F63" s="242"/>
-      <c r="G63" s="242"/>
-      <c r="H63" s="242"/>
-      <c r="I63" s="242"/>
-      <c r="J63" s="242"/>
-      <c r="K63" s="242"/>
-      <c r="L63" s="242"/>
-      <c r="M63" s="242"/>
-      <c r="N63" s="242"/>
+      <c r="C63" s="238"/>
+      <c r="D63" s="238"/>
+      <c r="E63" s="238"/>
+      <c r="F63" s="238"/>
+      <c r="G63" s="238"/>
+      <c r="H63" s="238"/>
+      <c r="I63" s="238"/>
+      <c r="J63" s="238"/>
+      <c r="K63" s="238"/>
+      <c r="L63" s="238"/>
+      <c r="M63" s="238"/>
+      <c r="N63" s="238"/>
     </row>
   </sheetData>
   <mergeCells count="17">
+    <mergeCell ref="A5:A6"/>
+    <mergeCell ref="B5:B6"/>
+    <mergeCell ref="C5:C6"/>
+    <mergeCell ref="D5:D6"/>
+    <mergeCell ref="E5:E6"/>
     <mergeCell ref="F5:F6"/>
     <mergeCell ref="C57:N63"/>
     <mergeCell ref="C54:N55"/>
@@ -7148,11 +7382,6 @@
     <mergeCell ref="L5:L6"/>
     <mergeCell ref="M5:M6"/>
     <mergeCell ref="I5:I6"/>
-    <mergeCell ref="A5:A6"/>
-    <mergeCell ref="B5:B6"/>
-    <mergeCell ref="C5:C6"/>
-    <mergeCell ref="D5:D6"/>
-    <mergeCell ref="E5:E6"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="landscape" r:id="rId1"/>

</xml_diff>